<commit_message>
Add Profitability + James comp-chart sheets to Capacity Lite
Profitability sheet: annual run-rate P&L comparing OLD vs NEW comp model
at the intake each one drives (old ~12/wk salary vs new ~25/wk
incentivized). Models commission payouts (James + reps, % of new signed
value) and MG&A overhead (fixed + variable %). Headline = delta net
profit ('profitability impact of the new comp model') with accretive/
dilutive verdict. All comp terms are editable inputs; notes document
assumptions.

James — New Comp sheet: change-management visual. Line chart of James's
annual pay OLD (flat salary) vs NEW (base + growth commission) across
intake levels, with crossover (~8/wk) and target (25/wk: +$61k) called
out. Linked to the Profitability inputs so it stays in sync.
</commit_message>
<xml_diff>
--- a/Capacity-Lite.xlsx
+++ b/Capacity-Lite.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Capacity Lite" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Profitability" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="James — New Comp" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,8 +115,64 @@
       <color rgb="00455064"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00101A30"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007A8499"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00101A30"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001B2A4A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00101A30"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C7415"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00101A30"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -150,8 +209,18 @@
         <fgColor rgb="00F6F8FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7EBF2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBECCB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -173,11 +242,80 @@
         <color rgb="00C2CAD8"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C2CAD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C2CAD8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C2CAD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C2CAD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C2CAD8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C2CAD8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C2CAD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C2CAD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C2CAD8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C2CAD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -265,12 +403,142 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="1"/>
@@ -306,6 +574,41 @@
           <fgColor rgb="00FBECCB"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002F7D5B"/>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9ECE2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B9831A"/>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBECCB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00B3402E"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002F7D5B"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -522,6 +825,165 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>James's annual pay: OLD (flat salary) vs NEW (base + growth commission)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'James — New Comp'!D11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="26000">
+              <a:solidFill>
+                <a:srgbClr val="1B2A4A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'James — New Comp'!$B$12:$B$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'James — New Comp'!$D$12:$D$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'James — New Comp'!E11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="34000">
+              <a:solidFill>
+                <a:srgbClr val="C8961E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'James — New Comp'!$B$12:$B$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'James — New Comp'!$E$12:$E$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>New cases signed per week</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>James pay ($/yr)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -532,6 +994,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3420000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1270,9 +1759,30 @@
         <f>IF(E23&gt;=E13,"ADD CAPACITY",IF(E23&lt;=E13-0.2,"SELL MORE","MAINTAIN"))</f>
         <v/>
       </c>
-    </row>
-    <row r="34" ht="24" customHeight="1"/>
-    <row r="35"/>
+      <c r="C33" s="30" t="n"/>
+      <c r="D33" s="30" t="n"/>
+      <c r="E33" s="30" t="n"/>
+      <c r="F33" s="30" t="n"/>
+      <c r="G33" s="30" t="n"/>
+      <c r="H33" s="30" t="n"/>
+      <c r="I33" s="30" t="n"/>
+      <c r="J33" s="31" t="n"/>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="B34" s="32" t="n"/>
+      <c r="J34" s="33" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="34" t="n"/>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="35" t="n"/>
+      <c r="F35" s="35" t="n"/>
+      <c r="G35" s="35" t="n"/>
+      <c r="H35" s="35" t="n"/>
+      <c r="I35" s="35" t="n"/>
+      <c r="J35" s="36" t="n"/>
+    </row>
     <row r="36">
       <c r="B36" s="19" t="inlineStr">
         <is>
@@ -1912,8 +2422,8 @@
     <mergeCell ref="F29:J29"/>
     <mergeCell ref="F11:J11"/>
     <mergeCell ref="B61:J61"/>
+    <mergeCell ref="B14:J14"/>
     <mergeCell ref="F10:J10"/>
-    <mergeCell ref="B14:J14"/>
     <mergeCell ref="F16:J16"/>
     <mergeCell ref="B60:J60"/>
     <mergeCell ref="F19:J19"/>
@@ -1977,4 +2487,1183 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F7D5B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="37" t="inlineStr">
+        <is>
+          <t>PROFITABILITY  ·  New Compensation Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="B3" s="38" t="inlineStr">
+        <is>
+          <t>Annual run-rate. Compares the OLD comp model vs the NEW (growth-incentive) model at the intake each one actually drives. Edit yellow (data) and blue (comp terms) cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Average case value ($)</t>
+        </is>
+      </c>
+      <c r="E6" s="41">
+        <f>'Capacity Lite'!E11</f>
+        <v/>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>linked from Capacity Lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Average case lifespan (months)</t>
+        </is>
+      </c>
+      <c r="E7" s="43">
+        <f>'Capacity Lite'!E12</f>
+        <v/>
+      </c>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>linked from Capacity Lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max active cases per manager</t>
+        </is>
+      </c>
+      <c r="E8" s="43">
+        <f>'Capacity Lite'!E16</f>
+        <v/>
+      </c>
+      <c r="G8" s="42" t="inlineStr">
+        <is>
+          <t>linked (≈143)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Collection rate (% of signed value)</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G9" s="42" t="inlineStr">
+        <is>
+          <t>share of signed fees actually collected</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intake UNDER OLD comp (cases/week)</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>what James/reps produce on salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intake UNDER NEW comp (cases/week)</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>the incentivized target: 3 reps + James</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James base — OLD ($/yr)</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>salary-heavy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James base — NEW ($/yr)</t>
+        </is>
+      </c>
+      <c r="E13" s="47" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G13" s="42" t="inlineStr">
+        <is>
+          <t>reduced base, upside from commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James commission — NEW (% of signed value)</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>growth commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Number of sales reps</t>
+        </is>
+      </c>
+      <c r="E15" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="42" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rep base — OLD ($/yr each)</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G16" s="42" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rep base — NEW ($/yr each)</t>
+        </is>
+      </c>
+      <c r="E17" s="47" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G17" s="42" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reps commission — NEW (% pooled)</t>
+        </is>
+      </c>
+      <c r="E18" s="48" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>across all reps, of signed value</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case manager loaded comp ($/yr)</t>
+        </is>
+      </c>
+      <c r="E19" s="50" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G19" s="42" t="inlineStr">
+        <is>
+          <t>delivery cost per manager FTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MG&amp;A overhead — fixed ($/yr)</t>
+        </is>
+      </c>
+      <c r="E20" s="50" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>rent, software, admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MG&amp;A overhead — variable (% of collected rev)</t>
+        </is>
+      </c>
+      <c r="E21" s="44" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>marketing / lead-gen scales with revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ANNUAL RUN-RATE P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="E24" s="53" t="inlineStr">
+        <is>
+          <t>OLD comp</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>NEW comp</t>
+        </is>
+      </c>
+      <c r="H24" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intake (cases/week)</t>
+        </is>
+      </c>
+      <c r="E25" s="55">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="G25" s="55">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="H25" s="42" t="inlineStr">
+        <is>
+          <t>behavioral: new comp lifts volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Annual signed case value</t>
+        </is>
+      </c>
+      <c r="E26" s="56">
+        <f>(E10*52*E6)</f>
+        <v/>
+      </c>
+      <c r="G26" s="56">
+        <f>(E11*52*E6)</f>
+        <v/>
+      </c>
+      <c r="H26" s="42" t="inlineStr">
+        <is>
+          <t>cases/wk × 52 × case value</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1">
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Collected revenue</t>
+        </is>
+      </c>
+      <c r="E27" s="56">
+        <f>(E10*52*E6)*E9</f>
+        <v/>
+      </c>
+      <c r="G27" s="56">
+        <f>(E11*52*E6)*E9</f>
+        <v/>
+      </c>
+      <c r="H27" s="42" t="inlineStr">
+        <is>
+          <t>signed × collection rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case managers required (FTE)</t>
+        </is>
+      </c>
+      <c r="E28" s="55">
+        <f>(E10*52*(E7/12))/E8</f>
+        <v/>
+      </c>
+      <c r="G28" s="55">
+        <f>(E11*52*(E7/12))/E8</f>
+        <v/>
+      </c>
+      <c r="H28" s="42" t="inlineStr">
+        <is>
+          <t>active cases ÷ max per mgr</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="19" customHeight="1">
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case manager cost</t>
+        </is>
+      </c>
+      <c r="E29" s="56">
+        <f>-((E10*52*(E7/12))/E8*E19)</f>
+        <v/>
+      </c>
+      <c r="G29" s="56">
+        <f>-((E11*52*(E7/12))/E8*E19)</f>
+        <v/>
+      </c>
+      <c r="H29" s="42" t="inlineStr">
+        <is>
+          <t>required FTE × loaded comp</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="B30" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James pay</t>
+        </is>
+      </c>
+      <c r="E30" s="56">
+        <f>-E12</f>
+        <v/>
+      </c>
+      <c r="G30" s="56">
+        <f>-(E13+E14*(E11*52*E6))</f>
+        <v/>
+      </c>
+      <c r="H30" s="42" t="inlineStr">
+        <is>
+          <t>OLD base  |  NEW base + commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sales reps pay</t>
+        </is>
+      </c>
+      <c r="E31" s="56">
+        <f>-(E15*E16)</f>
+        <v/>
+      </c>
+      <c r="G31" s="56">
+        <f>-(E15*E17+E18*(E11*52*E6))</f>
+        <v/>
+      </c>
+      <c r="H31" s="42" t="inlineStr">
+        <is>
+          <t>OLD base  |  NEW base + pooled commission</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="B32" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MG&amp;A overhead</t>
+        </is>
+      </c>
+      <c r="E32" s="56">
+        <f>-(E20+E21*((E10*52*E6)*E9))</f>
+        <v/>
+      </c>
+      <c r="G32" s="56">
+        <f>-(E20+E21*((E11*52*E6)*E9))</f>
+        <v/>
+      </c>
+      <c r="H32" s="42" t="inlineStr">
+        <is>
+          <t>fixed + variable % of collected rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1">
+      <c r="B33" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NET PROFIT</t>
+        </is>
+      </c>
+      <c r="E33" s="58">
+        <f>(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
+        <v/>
+      </c>
+      <c r="G33" s="58">
+        <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))</f>
+        <v/>
+      </c>
+      <c r="H33" s="42" t="inlineStr">
+        <is>
+          <t>collected rev − all costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="19" customHeight="1">
+      <c r="B34" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Net margin</t>
+        </is>
+      </c>
+      <c r="E34" s="59">
+        <f>(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))/((E10*52*E6)*E9)</f>
+        <v/>
+      </c>
+      <c r="G34" s="59">
+        <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))/((E11*52*E6)*E9)</f>
+        <v/>
+      </c>
+      <c r="H34" s="42" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="B36" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PROFITABILITY IMPACT OF THE NEW COMP MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ Collected revenue (new − old)</t>
+        </is>
+      </c>
+      <c r="E37" s="56">
+        <f>((E11*52*E6)*E9)-((E10*52*E6)*E9)</f>
+        <v/>
+      </c>
+      <c r="G37" s="62" t="inlineStr">
+        <is>
+          <t>the growth the incentive unlocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="B38" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ Selling comp cost (new − old)</t>
+        </is>
+      </c>
+      <c r="E38" s="56">
+        <f>-(((E13+E14*(E11*52*E6))+(E15*E17+E18*(E11*52*E6)))-(E12+(E15*E16)))</f>
+        <v/>
+      </c>
+      <c r="G38" s="62" t="inlineStr">
+        <is>
+          <t>extra commission the firm pays out</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Δ NET PROFIT (new − old)</t>
+        </is>
+      </c>
+      <c r="E39" s="64">
+        <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))-(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
+        <v/>
+      </c>
+      <c r="G39" s="62" t="inlineStr">
+        <is>
+          <t>bottom-line effect of switching</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="65">
+        <f>IF(E39&gt;=0,"NEW COMP MODEL IS ACCRETIVE — pays for itself through growth","NEW COMP COSTS MORE — justify via the added revenue &amp; retention")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>•  Commission basis = NEW SIGNED case value (rewards growth). James responds to visuals — see the 'James — New Comp' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="B46" s="29" t="inlineStr">
+        <is>
+          <t>•  The comparison is intentionally apples-to-oranges on VOLUME: the whole point of the new model is that it lifts intake (old ≈12/wk → new ≈25/wk). Set both intake cells to the same number to isolate the pure cost swap instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="B47" s="29" t="inlineStr">
+        <is>
+          <t>•  Run-rate view: at steady state, annual signed value ≈ annual recognized revenue. During rapid ramp, commission (paid on signings) leads revenue — watch cash timing separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>•  MG&amp;A variable % should include marketing / lead-gen (often the largest cost in tax resolution). Placeholder 30% — replace with actuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="B49" s="29" t="inlineStr">
+        <is>
+          <t>•  Collection rate accounts for refunds / non-payment. Placeholder 85%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="B50" s="29" t="inlineStr">
+        <is>
+          <t>•  All comp terms are placeholders pending David's real numbers — every one is an editable input.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="43">
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="H27"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B49:H49"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="H33"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="H30"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="H26"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="H29"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="B47:H47"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B46:H46"/>
+    <mergeCell ref="H31"/>
+    <mergeCell ref="H25"/>
+    <mergeCell ref="H34"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="B48:H48"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="H32"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="B41:H42"/>
+    <mergeCell ref="H28"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B41">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>E39&gt;=0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="4">
+      <formula>E39&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:E34">
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>E25&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25:G34">
+    <cfRule type="expression" priority="4" dxfId="5">
+      <formula>G25&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C8961E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="37" t="inlineStr">
+        <is>
+          <t>WHY THE NEW MODEL PAYS JAMES MORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="66" t="inlineStr">
+        <is>
+          <t>Old model = flat salary no matter how much the firm grows. New model = lower base + commission on new signed cases, so his pay climbs with the growth he drives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James base — OLD</t>
+        </is>
+      </c>
+      <c r="C5" s="67">
+        <f>'Profitability'!E12</f>
+        <v/>
+      </c>
+      <c r="E5" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Target intake (cases/wk)</t>
+        </is>
+      </c>
+      <c r="F5" s="68">
+        <f>'Profitability'!E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  James base — NEW</t>
+        </is>
+      </c>
+      <c r="C6" s="69">
+        <f>'Profitability'!E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Commission % (signed value)</t>
+        </is>
+      </c>
+      <c r="C7" s="70">
+        <f>'Profitability'!E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case value</t>
+        </is>
+      </c>
+      <c r="C8" s="71">
+        <f>'Profitability'!E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="72" t="inlineStr">
+        <is>
+          <t>Cases / week</t>
+        </is>
+      </c>
+      <c r="C11" s="72" t="inlineStr">
+        <is>
+          <t>Signed value / yr</t>
+        </is>
+      </c>
+      <c r="D11" s="72" t="inlineStr">
+        <is>
+          <t>James OLD ($)</t>
+        </is>
+      </c>
+      <c r="E11" s="72" t="inlineStr">
+        <is>
+          <t>James NEW ($)</t>
+        </is>
+      </c>
+      <c r="F11" s="72" t="inlineStr">
+        <is>
+          <t>Δ to James</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="B12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="56">
+        <f>B12*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D12" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E12" s="73">
+        <f>$C$6+$C$7*C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="56">
+        <f>E12-D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="55" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C13" s="56">
+        <f>B13*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D13" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E13" s="73">
+        <f>$C$6+$C$7*C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="56">
+        <f>E13-D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="B14" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="56">
+        <f>B14*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D14" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E14" s="73">
+        <f>$C$6+$C$7*C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="56">
+        <f>E14-D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="B15" s="55" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C15" s="56">
+        <f>B15*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D15" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E15" s="73">
+        <f>$C$6+$C$7*C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="56">
+        <f>E15-D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="56">
+        <f>B16*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D16" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E16" s="73">
+        <f>$C$6+$C$7*C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="56">
+        <f>E16-D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="B17" s="55" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C17" s="56">
+        <f>B17*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D17" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E17" s="73">
+        <f>$C$6+$C$7*C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="56">
+        <f>E17-D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="B18" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" s="56">
+        <f>B18*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E18" s="73">
+        <f>$C$6+$C$7*C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="56">
+        <f>E18-D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="B19" s="55" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="C19" s="56">
+        <f>B19*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D19" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E19" s="73">
+        <f>$C$6+$C$7*C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="56">
+        <f>E19-D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="B20" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" s="56">
+        <f>B20*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D20" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E20" s="73">
+        <f>$C$6+$C$7*C20</f>
+        <v/>
+      </c>
+      <c r="F20" s="56">
+        <f>E20-D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="B21" s="55" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C21" s="56">
+        <f>B21*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D21" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E21" s="73">
+        <f>$C$6+$C$7*C21</f>
+        <v/>
+      </c>
+      <c r="F21" s="56">
+        <f>E21-D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="74" t="n">
+        <v>25</v>
+      </c>
+      <c r="C22" s="75">
+        <f>B22*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="75">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E22" s="75">
+        <f>$C$6+$C$7*C22</f>
+        <v/>
+      </c>
+      <c r="F22" s="75">
+        <f>E22-D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="55" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="C23" s="56">
+        <f>B23*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D23" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E23" s="73">
+        <f>$C$6+$C$7*C23</f>
+        <v/>
+      </c>
+      <c r="F23" s="56">
+        <f>E23-D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="C24" s="56">
+        <f>B24*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D24" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E24" s="73">
+        <f>$C$6+$C$7*C24</f>
+        <v/>
+      </c>
+      <c r="F24" s="56">
+        <f>E24-D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="B25" s="55" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="C25" s="56">
+        <f>B25*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D25" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E25" s="73">
+        <f>$C$6+$C$7*C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="56">
+        <f>E25-D25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="B26" s="55" t="n">
+        <v>35</v>
+      </c>
+      <c r="C26" s="56">
+        <f>B26*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D26" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E26" s="73">
+        <f>$C$6+$C$7*C26</f>
+        <v/>
+      </c>
+      <c r="F26" s="56">
+        <f>E26-D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="B27" s="55" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C27" s="56">
+        <f>B27*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D27" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E27" s="73">
+        <f>$C$6+$C$7*C27</f>
+        <v/>
+      </c>
+      <c r="F27" s="56">
+        <f>E27-D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="55" t="n">
+        <v>40</v>
+      </c>
+      <c r="C28" s="56">
+        <f>B28*52*$C$8</f>
+        <v/>
+      </c>
+      <c r="D28" s="56">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="E28" s="73">
+        <f>$C$6+$C$7*C28</f>
+        <v/>
+      </c>
+      <c r="F28" s="56">
+        <f>E28-D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="76">
+        <f>CONCATENATE("At the ",TEXT($F$5,"0")," cases/week goal: OLD ",TEXT(D22,"$#,##0")," → NEW ",TEXT(E22,"$#,##0")," (",TEXT(F22,"+$#,##0"),"/yr for James)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="77" t="inlineStr">
+        <is>
+          <t>The lines cross near ~8 cases/week — beyond that, James earns more under the new model, and it keeps climbing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F12:F28">
+    <cfRule type="expression" priority="1" dxfId="6">
+      <formula>F12&gt;=0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="5">
+      <formula>F12&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Cash Timing and Comp Optimizer sheets to Capacity Lite
Cash Timing: 18-month cash projection modeling commission paid up front
on signings vs fees collected over the case lifespan. Surfaces the ramp
gap between run-rate profit and actual early-month cash, flags the
cumulative-cash trough and whether it goes negative.

Comp Optimizer: solves for the highest James commission % that (a) keeps
the firm no worse than the old model and (b) holds a target net margin,
with a sensitivity table and a net-profit-vs-rate chart against the
old-model reference line. All linked to the Profitability inputs.
</commit_message>
<xml_diff>
--- a/Capacity-Lite.xlsx
+++ b/Capacity-Lite.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Capacity Lite" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Profitability" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="James — New Comp" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Timing" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Comp Optimizer" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -171,6 +173,34 @@
       <b val="1"/>
       <color rgb="00101A30"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00B3402E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002F7D5B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00101A30"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -220,7 +250,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -311,11 +341,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C2CAD8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C2CAD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C2CAD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C2CAD8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C2CAD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -534,11 +588,127 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="12">
     <dxf>
       <font>
         <b val="1"/>
@@ -609,6 +779,57 @@
         <b val="1"/>
         <color rgb="002F7D5B"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B3402E"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B3402E"/>
+        <sz val="13"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4D8D1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002F7D5B"/>
+        <sz val="13"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9ECE2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002F7D5B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9ECE2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00B3402E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4D8D1"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -984,6 +1205,432 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumulative cash through the ramp</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cash Timing'!J22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="32000">
+              <a:solidFill>
+                <a:srgbClr val="1B2A4A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cash Timing'!$B$23:$B$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cash Timing'!$J$23:$J$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cash</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly collections vs run-rate revenue vs commission paid</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cash Timing'!F22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="30000">
+              <a:solidFill>
+                <a:srgbClr val="2F7D5B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cash Timing'!$B$23:$B$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cash Timing'!$F$23:$F$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cash Timing'!K22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C8961E"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cash Timing'!$B$23:$B$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cash Timing'!$K$23:$K$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Cash Timing'!D22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B3402E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cash Timing'!$B$23:$B$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cash Timing'!$D$23:$D$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Firm net profit vs James commission % (break-even where it meets the old-model line)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Comp Optimizer'!D16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="32000">
+              <a:solidFill>
+                <a:srgbClr val="C8961E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Comp Optimizer'!$B$17:$B$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comp Optimizer'!$D$17:$D$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Comp Optimizer'!G16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1B2A4A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Comp Optimizer'!$B$17:$B$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comp Optimizer'!$G$17:$G$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>James commission %</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Firm net profit</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1021,6 +1668,82 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1345,28 +2068,28 @@
   </cols>
   <sheetData>
     <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="37" t="inlineStr">
         <is>
           <t>CAPACITY LITE  ·  Tax Resolution  ·  Revenue-Based (v2)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>Capacity is a REVENUE ceiling per case manager; case counts are derived. Edit the yellow (team/data) and blue (David's model definitions) cells.  Model owner: David.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  INPUTS</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Full-capacity case managers (FTE)</t>
         </is>
@@ -1381,7 +2104,7 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case managers in training (count)</t>
         </is>
@@ -1396,7 +2119,7 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Current active (open) cases</t>
         </is>
@@ -1411,7 +2134,7 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  New cases signed / week</t>
         </is>
@@ -1426,7 +2149,7 @@
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue capacity per manager ($/yr)</t>
         </is>
@@ -1441,7 +2164,7 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case value ($)</t>
         </is>
@@ -1456,7 +2179,7 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case lifespan (months)</t>
         </is>
@@ -1471,7 +2194,7 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfort ceiling (% of capacity)</t>
         </is>
@@ -1486,14 +2209,14 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  DERIVED CAPACITY</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Effective case managers (FTE)</t>
         </is>
@@ -1509,7 +2232,7 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Max active cases per manager</t>
         </is>
@@ -1525,7 +2248,7 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total revenue capacity</t>
         </is>
@@ -1541,7 +2264,7 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total case capacity</t>
         </is>
@@ -1557,7 +2280,7 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfortable revenue capacity</t>
         </is>
@@ -1573,7 +2296,7 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Historical benchmark (cases/mgr, w/ admin)</t>
         </is>
@@ -1588,14 +2311,14 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  CURRENT STATE</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Current active book value</t>
         </is>
@@ -1611,7 +2334,7 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue utilization</t>
         </is>
@@ -1627,7 +2350,7 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Headroom to comfort ($)</t>
         </is>
@@ -1643,7 +2366,7 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Headroom to comfort (cases)</t>
         </is>
@@ -1659,7 +2382,7 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  New cases / month</t>
         </is>
@@ -1675,7 +2398,7 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cases closing / month</t>
         </is>
@@ -1691,7 +2414,7 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Net case growth / month</t>
         </is>
@@ -1707,7 +2430,7 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Net revenue growth / month</t>
         </is>
@@ -1723,7 +2446,7 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Months to comfortably full</t>
         </is>
@@ -1739,7 +2462,7 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Implied annual revenue throughput</t>
         </is>
@@ -1784,14 +2507,14 @@
       <c r="J35" s="36" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B36" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">  Three states: at/above the comfort ceiling → ADD CAPACITY · more than 20 pts below → SELL MORE · in between → MAINTAIN.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  12-MONTH PROJECTION  (assumes intake, case value &amp; lifespan hold steady)</t>
         </is>
@@ -1869,7 +2592,7 @@
         <f>E8</f>
         <v/>
       </c>
-      <c r="G39" s="24">
+      <c r="G39" s="56">
         <f>F39*$E$11</f>
         <v/>
       </c>
@@ -1892,15 +2615,15 @@
           <t>Mo 1</t>
         </is>
       </c>
-      <c r="C40" s="28">
+      <c r="C40" s="55">
         <f>F39</f>
         <v/>
       </c>
-      <c r="D40" s="28">
+      <c r="D40" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E40" s="28">
+      <c r="E40" s="55">
         <f>C40/$E$12</f>
         <v/>
       </c>
@@ -1908,7 +2631,7 @@
         <f>MAX(0,C40+D40-E40)</f>
         <v/>
       </c>
-      <c r="G40" s="24">
+      <c r="G40" s="56">
         <f>F40*$E$11</f>
         <v/>
       </c>
@@ -1931,15 +2654,15 @@
           <t>Mo 2</t>
         </is>
       </c>
-      <c r="C41" s="28">
+      <c r="C41" s="55">
         <f>F40</f>
         <v/>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E41" s="28">
+      <c r="E41" s="55">
         <f>C41/$E$12</f>
         <v/>
       </c>
@@ -1947,7 +2670,7 @@
         <f>MAX(0,C41+D41-E41)</f>
         <v/>
       </c>
-      <c r="G41" s="24">
+      <c r="G41" s="56">
         <f>F41*$E$11</f>
         <v/>
       </c>
@@ -1970,15 +2693,15 @@
           <t>Mo 3</t>
         </is>
       </c>
-      <c r="C42" s="28">
+      <c r="C42" s="55">
         <f>F41</f>
         <v/>
       </c>
-      <c r="D42" s="28">
+      <c r="D42" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E42" s="28">
+      <c r="E42" s="55">
         <f>C42/$E$12</f>
         <v/>
       </c>
@@ -1986,7 +2709,7 @@
         <f>MAX(0,C42+D42-E42)</f>
         <v/>
       </c>
-      <c r="G42" s="24">
+      <c r="G42" s="56">
         <f>F42*$E$11</f>
         <v/>
       </c>
@@ -2009,15 +2732,15 @@
           <t>Mo 4</t>
         </is>
       </c>
-      <c r="C43" s="28">
+      <c r="C43" s="55">
         <f>F42</f>
         <v/>
       </c>
-      <c r="D43" s="28">
+      <c r="D43" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E43" s="28">
+      <c r="E43" s="55">
         <f>C43/$E$12</f>
         <v/>
       </c>
@@ -2025,7 +2748,7 @@
         <f>MAX(0,C43+D43-E43)</f>
         <v/>
       </c>
-      <c r="G43" s="24">
+      <c r="G43" s="56">
         <f>F43*$E$11</f>
         <v/>
       </c>
@@ -2048,15 +2771,15 @@
           <t>Mo 5</t>
         </is>
       </c>
-      <c r="C44" s="28">
+      <c r="C44" s="55">
         <f>F43</f>
         <v/>
       </c>
-      <c r="D44" s="28">
+      <c r="D44" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E44" s="28">
+      <c r="E44" s="55">
         <f>C44/$E$12</f>
         <v/>
       </c>
@@ -2064,7 +2787,7 @@
         <f>MAX(0,C44+D44-E44)</f>
         <v/>
       </c>
-      <c r="G44" s="24">
+      <c r="G44" s="56">
         <f>F44*$E$11</f>
         <v/>
       </c>
@@ -2087,15 +2810,15 @@
           <t>Mo 6</t>
         </is>
       </c>
-      <c r="C45" s="28">
+      <c r="C45" s="55">
         <f>F44</f>
         <v/>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E45" s="28">
+      <c r="E45" s="55">
         <f>C45/$E$12</f>
         <v/>
       </c>
@@ -2103,7 +2826,7 @@
         <f>MAX(0,C45+D45-E45)</f>
         <v/>
       </c>
-      <c r="G45" s="24">
+      <c r="G45" s="56">
         <f>F45*$E$11</f>
         <v/>
       </c>
@@ -2126,15 +2849,15 @@
           <t>Mo 7</t>
         </is>
       </c>
-      <c r="C46" s="28">
+      <c r="C46" s="55">
         <f>F45</f>
         <v/>
       </c>
-      <c r="D46" s="28">
+      <c r="D46" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E46" s="28">
+      <c r="E46" s="55">
         <f>C46/$E$12</f>
         <v/>
       </c>
@@ -2142,7 +2865,7 @@
         <f>MAX(0,C46+D46-E46)</f>
         <v/>
       </c>
-      <c r="G46" s="24">
+      <c r="G46" s="56">
         <f>F46*$E$11</f>
         <v/>
       </c>
@@ -2165,15 +2888,15 @@
           <t>Mo 8</t>
         </is>
       </c>
-      <c r="C47" s="28">
+      <c r="C47" s="55">
         <f>F46</f>
         <v/>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E47" s="28">
+      <c r="E47" s="55">
         <f>C47/$E$12</f>
         <v/>
       </c>
@@ -2181,7 +2904,7 @@
         <f>MAX(0,C47+D47-E47)</f>
         <v/>
       </c>
-      <c r="G47" s="24">
+      <c r="G47" s="56">
         <f>F47*$E$11</f>
         <v/>
       </c>
@@ -2204,15 +2927,15 @@
           <t>Mo 9</t>
         </is>
       </c>
-      <c r="C48" s="28">
+      <c r="C48" s="55">
         <f>F47</f>
         <v/>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E48" s="28">
+      <c r="E48" s="55">
         <f>C48/$E$12</f>
         <v/>
       </c>
@@ -2220,7 +2943,7 @@
         <f>MAX(0,C48+D48-E48)</f>
         <v/>
       </c>
-      <c r="G48" s="24">
+      <c r="G48" s="56">
         <f>F48*$E$11</f>
         <v/>
       </c>
@@ -2243,15 +2966,15 @@
           <t>Mo 10</t>
         </is>
       </c>
-      <c r="C49" s="28">
+      <c r="C49" s="55">
         <f>F48</f>
         <v/>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E49" s="28">
+      <c r="E49" s="55">
         <f>C49/$E$12</f>
         <v/>
       </c>
@@ -2259,7 +2982,7 @@
         <f>MAX(0,C49+D49-E49)</f>
         <v/>
       </c>
-      <c r="G49" s="24">
+      <c r="G49" s="56">
         <f>F49*$E$11</f>
         <v/>
       </c>
@@ -2282,15 +3005,15 @@
           <t>Mo 11</t>
         </is>
       </c>
-      <c r="C50" s="28">
+      <c r="C50" s="55">
         <f>F49</f>
         <v/>
       </c>
-      <c r="D50" s="28">
+      <c r="D50" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E50" s="28">
+      <c r="E50" s="55">
         <f>C50/$E$12</f>
         <v/>
       </c>
@@ -2298,7 +3021,7 @@
         <f>MAX(0,C50+D50-E50)</f>
         <v/>
       </c>
-      <c r="G50" s="24">
+      <c r="G50" s="56">
         <f>F50*$E$11</f>
         <v/>
       </c>
@@ -2321,15 +3044,15 @@
           <t>Mo 12</t>
         </is>
       </c>
-      <c r="C51" s="28">
+      <c r="C51" s="55">
         <f>F50</f>
         <v/>
       </c>
-      <c r="D51" s="28">
+      <c r="D51" s="55">
         <f>$E$26</f>
         <v/>
       </c>
-      <c r="E51" s="28">
+      <c r="E51" s="55">
         <f>C51/$E$12</f>
         <v/>
       </c>
@@ -2337,7 +3060,7 @@
         <f>MAX(0,C51+D51-E51)</f>
         <v/>
       </c>
-      <c r="G51" s="24">
+      <c r="G51" s="56">
         <f>F51*$E$11</f>
         <v/>
       </c>
@@ -2355,7 +3078,7 @@
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B53" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
         </is>
@@ -3046,8 +3769,22 @@
         <f>IF(E39&gt;=0,"NEW COMP MODEL IS ACCRETIVE — pays for itself through growth","NEW COMP COSTS MORE — justify via the added revenue &amp; retention")</f>
         <v/>
       </c>
-    </row>
-    <row r="42"/>
+      <c r="C41" s="30" t="n"/>
+      <c r="D41" s="30" t="n"/>
+      <c r="E41" s="30" t="n"/>
+      <c r="F41" s="30" t="n"/>
+      <c r="G41" s="30" t="n"/>
+      <c r="H41" s="31" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="34" t="n"/>
+      <c r="C42" s="35" t="n"/>
+      <c r="D42" s="35" t="n"/>
+      <c r="E42" s="35" t="n"/>
+      <c r="F42" s="35" t="n"/>
+      <c r="G42" s="35" t="n"/>
+      <c r="H42" s="36" t="n"/>
+    </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="51" t="inlineStr">
         <is>
@@ -3100,8 +3837,8 @@
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="G21:H21"/>
+    <mergeCell ref="H27"/>
     <mergeCell ref="G12:H12"/>
-    <mergeCell ref="H27"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="B49:H49"/>
     <mergeCell ref="G11:H11"/>
@@ -3640,6 +4377,10 @@
         <f>CONCATENATE("At the ",TEXT($F$5,"0")," cases/week goal: OLD ",TEXT(D22,"$#,##0")," → NEW ",TEXT(E22,"$#,##0")," (",TEXT(F22,"+$#,##0"),"/yr for James)")</f>
         <v/>
       </c>
+      <c r="C30" s="78" t="n"/>
+      <c r="D30" s="78" t="n"/>
+      <c r="E30" s="78" t="n"/>
+      <c r="F30" s="79" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="77" t="inlineStr">
@@ -3666,4 +4407,1628 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00B3402E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:K46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="80" t="inlineStr">
+        <is>
+          <t>CASH TIMING  ·  Why the Ramp Pinches</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="B3" s="81" t="inlineStr">
+        <is>
+          <t>Commission is paid up front on signings, but fees collect over the case lifespan. Early months bank far less cash than the run-rate P&amp;L implies. 18-month view at the NEW-comp intake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DRIVERS (linked from Profitability / Capacity Lite; yellow = editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Starting cash ($)</t>
+        </is>
+      </c>
+      <c r="F6" s="84" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Starting open book (cases)</t>
+        </is>
+      </c>
+      <c r="F7" s="85">
+        <f>'Capacity Lite'!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Intake (cases / month)</t>
+        </is>
+      </c>
+      <c r="F8" s="86">
+        <f>'Profitability'!E11*52/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case value ($)</t>
+        </is>
+      </c>
+      <c r="F9" s="87">
+        <f>'Profitability'!E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lifespan (months)</t>
+        </is>
+      </c>
+      <c r="F10" s="86">
+        <f>'Profitability'!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Collection rate</t>
+        </is>
+      </c>
+      <c r="F11" s="88">
+        <f>'Profitability'!E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total commission rate (James+reps)</t>
+        </is>
+      </c>
+      <c r="F12" s="89">
+        <f>'Profitability'!E14+'Profitability'!E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base comp — James+reps / month</t>
+        </is>
+      </c>
+      <c r="F13" s="87">
+        <f>('Profitability'!E13+'Profitability'!E15*'Profitability'!E17)/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max cases / mgr</t>
+        </is>
+      </c>
+      <c r="F14" s="86">
+        <f>'Profitability'!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case mgr loaded comp ($/yr)</t>
+        </is>
+      </c>
+      <c r="F15" s="87">
+        <f>'Profitability'!E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MG&amp;A fixed / month</t>
+        </is>
+      </c>
+      <c r="F16" s="87">
+        <f>'Profitability'!E20/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MG&amp;A variable (% of collections)</t>
+        </is>
+      </c>
+      <c r="F17" s="88">
+        <f>'Profitability'!E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Collection per active case / month</t>
+        </is>
+      </c>
+      <c r="F18" s="90">
+        <f>F9*F11/F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Run-rate collected revenue / month (steady state)</t>
+        </is>
+      </c>
+      <c r="F19" s="90">
+        <f>F8*F9*F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  18-MONTH CASH PROJECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="B22" s="92" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C22" s="92" t="inlineStr">
+        <is>
+          <t>New signings $</t>
+        </is>
+      </c>
+      <c r="D22" s="92" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="E22" s="92" t="inlineStr">
+        <is>
+          <t>Active cases</t>
+        </is>
+      </c>
+      <c r="F22" s="92" t="inlineStr">
+        <is>
+          <t>Collections</t>
+        </is>
+      </c>
+      <c r="G22" s="92" t="inlineStr">
+        <is>
+          <t>Case mgr cost</t>
+        </is>
+      </c>
+      <c r="H22" s="92" t="inlineStr">
+        <is>
+          <t>Base + MG&amp;A</t>
+        </is>
+      </c>
+      <c r="I22" s="92" t="inlineStr">
+        <is>
+          <t>Net cash</t>
+        </is>
+      </c>
+      <c r="J22" s="92" t="inlineStr">
+        <is>
+          <t>Cumulative cash</t>
+        </is>
+      </c>
+      <c r="K22" s="92" t="inlineStr">
+        <is>
+          <t>Run-rate rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D23" s="95">
+        <f>F12*C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="96">
+        <f>F7*MAX(0,(F10-(1-1))/F10)+F8*MIN(1,F10)</f>
+        <v/>
+      </c>
+      <c r="F23" s="97">
+        <f>E23*F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="94">
+        <f>E23/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H23" s="94">
+        <f>F13+F16+F17*F23</f>
+        <v/>
+      </c>
+      <c r="I23" s="98">
+        <f>F23-D23-G23-H23</f>
+        <v/>
+      </c>
+      <c r="J23" s="99">
+        <f>F6+I23</f>
+        <v/>
+      </c>
+      <c r="K23" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D24" s="95">
+        <f>F12*C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="96">
+        <f>F7*MAX(0,(F10-(2-1))/F10)+F8*MIN(2,F10)</f>
+        <v/>
+      </c>
+      <c r="F24" s="97">
+        <f>E24*F18</f>
+        <v/>
+      </c>
+      <c r="G24" s="94">
+        <f>E24/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H24" s="94">
+        <f>F13+F16+F17*F24</f>
+        <v/>
+      </c>
+      <c r="I24" s="98">
+        <f>F24-D24-G24-H24</f>
+        <v/>
+      </c>
+      <c r="J24" s="99">
+        <f>J23+I24</f>
+        <v/>
+      </c>
+      <c r="K24" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="93" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D25" s="95">
+        <f>F12*C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="96">
+        <f>F7*MAX(0,(F10-(3-1))/F10)+F8*MIN(3,F10)</f>
+        <v/>
+      </c>
+      <c r="F25" s="97">
+        <f>E25*F18</f>
+        <v/>
+      </c>
+      <c r="G25" s="94">
+        <f>E25/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H25" s="94">
+        <f>F13+F16+F17*F25</f>
+        <v/>
+      </c>
+      <c r="I25" s="98">
+        <f>F25-D25-G25-H25</f>
+        <v/>
+      </c>
+      <c r="J25" s="99">
+        <f>J24+I25</f>
+        <v/>
+      </c>
+      <c r="K25" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="93" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D26" s="95">
+        <f>F12*C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="96">
+        <f>F7*MAX(0,(F10-(4-1))/F10)+F8*MIN(4,F10)</f>
+        <v/>
+      </c>
+      <c r="F26" s="97">
+        <f>E26*F18</f>
+        <v/>
+      </c>
+      <c r="G26" s="94">
+        <f>E26/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H26" s="94">
+        <f>F13+F16+F17*F26</f>
+        <v/>
+      </c>
+      <c r="I26" s="98">
+        <f>F26-D26-G26-H26</f>
+        <v/>
+      </c>
+      <c r="J26" s="99">
+        <f>J25+I26</f>
+        <v/>
+      </c>
+      <c r="K26" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="B27" s="93" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D27" s="95">
+        <f>F12*C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="96">
+        <f>F7*MAX(0,(F10-(5-1))/F10)+F8*MIN(5,F10)</f>
+        <v/>
+      </c>
+      <c r="F27" s="97">
+        <f>E27*F18</f>
+        <v/>
+      </c>
+      <c r="G27" s="94">
+        <f>E27/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H27" s="94">
+        <f>F13+F16+F17*F27</f>
+        <v/>
+      </c>
+      <c r="I27" s="98">
+        <f>F27-D27-G27-H27</f>
+        <v/>
+      </c>
+      <c r="J27" s="99">
+        <f>J26+I27</f>
+        <v/>
+      </c>
+      <c r="K27" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="B28" s="93" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D28" s="95">
+        <f>F12*C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="96">
+        <f>F7*MAX(0,(F10-(6-1))/F10)+F8*MIN(6,F10)</f>
+        <v/>
+      </c>
+      <c r="F28" s="97">
+        <f>E28*F18</f>
+        <v/>
+      </c>
+      <c r="G28" s="94">
+        <f>E28/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H28" s="94">
+        <f>F13+F16+F17*F28</f>
+        <v/>
+      </c>
+      <c r="I28" s="98">
+        <f>F28-D28-G28-H28</f>
+        <v/>
+      </c>
+      <c r="J28" s="99">
+        <f>J27+I28</f>
+        <v/>
+      </c>
+      <c r="K28" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="B29" s="93" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D29" s="95">
+        <f>F12*C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="96">
+        <f>F7*MAX(0,(F10-(7-1))/F10)+F8*MIN(7,F10)</f>
+        <v/>
+      </c>
+      <c r="F29" s="97">
+        <f>E29*F18</f>
+        <v/>
+      </c>
+      <c r="G29" s="94">
+        <f>E29/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H29" s="94">
+        <f>F13+F16+F17*F29</f>
+        <v/>
+      </c>
+      <c r="I29" s="98">
+        <f>F29-D29-G29-H29</f>
+        <v/>
+      </c>
+      <c r="J29" s="99">
+        <f>J28+I29</f>
+        <v/>
+      </c>
+      <c r="K29" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="B30" s="93" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D30" s="95">
+        <f>F12*C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="96">
+        <f>F7*MAX(0,(F10-(8-1))/F10)+F8*MIN(8,F10)</f>
+        <v/>
+      </c>
+      <c r="F30" s="97">
+        <f>E30*F18</f>
+        <v/>
+      </c>
+      <c r="G30" s="94">
+        <f>E30/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H30" s="94">
+        <f>F13+F16+F17*F30</f>
+        <v/>
+      </c>
+      <c r="I30" s="98">
+        <f>F30-D30-G30-H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="99">
+        <f>J29+I30</f>
+        <v/>
+      </c>
+      <c r="K30" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="B31" s="93" t="n">
+        <v>9</v>
+      </c>
+      <c r="C31" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D31" s="95">
+        <f>F12*C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="96">
+        <f>F7*MAX(0,(F10-(9-1))/F10)+F8*MIN(9,F10)</f>
+        <v/>
+      </c>
+      <c r="F31" s="97">
+        <f>E31*F18</f>
+        <v/>
+      </c>
+      <c r="G31" s="94">
+        <f>E31/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H31" s="94">
+        <f>F13+F16+F17*F31</f>
+        <v/>
+      </c>
+      <c r="I31" s="98">
+        <f>F31-D31-G31-H31</f>
+        <v/>
+      </c>
+      <c r="J31" s="99">
+        <f>J30+I31</f>
+        <v/>
+      </c>
+      <c r="K31" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="B32" s="93" t="n">
+        <v>10</v>
+      </c>
+      <c r="C32" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D32" s="95">
+        <f>F12*C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="96">
+        <f>F7*MAX(0,(F10-(10-1))/F10)+F8*MIN(10,F10)</f>
+        <v/>
+      </c>
+      <c r="F32" s="97">
+        <f>E32*F18</f>
+        <v/>
+      </c>
+      <c r="G32" s="94">
+        <f>E32/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H32" s="94">
+        <f>F13+F16+F17*F32</f>
+        <v/>
+      </c>
+      <c r="I32" s="98">
+        <f>F32-D32-G32-H32</f>
+        <v/>
+      </c>
+      <c r="J32" s="99">
+        <f>J31+I32</f>
+        <v/>
+      </c>
+      <c r="K32" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="B33" s="93" t="n">
+        <v>11</v>
+      </c>
+      <c r="C33" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D33" s="95">
+        <f>F12*C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="96">
+        <f>F7*MAX(0,(F10-(11-1))/F10)+F8*MIN(11,F10)</f>
+        <v/>
+      </c>
+      <c r="F33" s="97">
+        <f>E33*F18</f>
+        <v/>
+      </c>
+      <c r="G33" s="94">
+        <f>E33/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H33" s="94">
+        <f>F13+F16+F17*F33</f>
+        <v/>
+      </c>
+      <c r="I33" s="98">
+        <f>F33-D33-G33-H33</f>
+        <v/>
+      </c>
+      <c r="J33" s="99">
+        <f>J32+I33</f>
+        <v/>
+      </c>
+      <c r="K33" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="B34" s="93" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D34" s="95">
+        <f>F12*C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="96">
+        <f>F7*MAX(0,(F10-(12-1))/F10)+F8*MIN(12,F10)</f>
+        <v/>
+      </c>
+      <c r="F34" s="97">
+        <f>E34*F18</f>
+        <v/>
+      </c>
+      <c r="G34" s="94">
+        <f>E34/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H34" s="94">
+        <f>F13+F16+F17*F34</f>
+        <v/>
+      </c>
+      <c r="I34" s="98">
+        <f>F34-D34-G34-H34</f>
+        <v/>
+      </c>
+      <c r="J34" s="99">
+        <f>J33+I34</f>
+        <v/>
+      </c>
+      <c r="K34" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="93" t="n">
+        <v>13</v>
+      </c>
+      <c r="C35" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D35" s="95">
+        <f>F12*C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="96">
+        <f>F7*MAX(0,(F10-(13-1))/F10)+F8*MIN(13,F10)</f>
+        <v/>
+      </c>
+      <c r="F35" s="97">
+        <f>E35*F18</f>
+        <v/>
+      </c>
+      <c r="G35" s="94">
+        <f>E35/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H35" s="94">
+        <f>F13+F16+F17*F35</f>
+        <v/>
+      </c>
+      <c r="I35" s="98">
+        <f>F35-D35-G35-H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="99">
+        <f>J34+I35</f>
+        <v/>
+      </c>
+      <c r="K35" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="B36" s="93" t="n">
+        <v>14</v>
+      </c>
+      <c r="C36" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D36" s="95">
+        <f>F12*C36</f>
+        <v/>
+      </c>
+      <c r="E36" s="96">
+        <f>F7*MAX(0,(F10-(14-1))/F10)+F8*MIN(14,F10)</f>
+        <v/>
+      </c>
+      <c r="F36" s="97">
+        <f>E36*F18</f>
+        <v/>
+      </c>
+      <c r="G36" s="94">
+        <f>E36/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H36" s="94">
+        <f>F13+F16+F17*F36</f>
+        <v/>
+      </c>
+      <c r="I36" s="98">
+        <f>F36-D36-G36-H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="99">
+        <f>J35+I36</f>
+        <v/>
+      </c>
+      <c r="K36" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="B37" s="93" t="n">
+        <v>15</v>
+      </c>
+      <c r="C37" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D37" s="95">
+        <f>F12*C37</f>
+        <v/>
+      </c>
+      <c r="E37" s="96">
+        <f>F7*MAX(0,(F10-(15-1))/F10)+F8*MIN(15,F10)</f>
+        <v/>
+      </c>
+      <c r="F37" s="97">
+        <f>E37*F18</f>
+        <v/>
+      </c>
+      <c r="G37" s="94">
+        <f>E37/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H37" s="94">
+        <f>F13+F16+F17*F37</f>
+        <v/>
+      </c>
+      <c r="I37" s="98">
+        <f>F37-D37-G37-H37</f>
+        <v/>
+      </c>
+      <c r="J37" s="99">
+        <f>J36+I37</f>
+        <v/>
+      </c>
+      <c r="K37" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="B38" s="93" t="n">
+        <v>16</v>
+      </c>
+      <c r="C38" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D38" s="95">
+        <f>F12*C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="96">
+        <f>F7*MAX(0,(F10-(16-1))/F10)+F8*MIN(16,F10)</f>
+        <v/>
+      </c>
+      <c r="F38" s="97">
+        <f>E38*F18</f>
+        <v/>
+      </c>
+      <c r="G38" s="94">
+        <f>E38/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H38" s="94">
+        <f>F13+F16+F17*F38</f>
+        <v/>
+      </c>
+      <c r="I38" s="98">
+        <f>F38-D38-G38-H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="99">
+        <f>J37+I38</f>
+        <v/>
+      </c>
+      <c r="K38" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="B39" s="93" t="n">
+        <v>17</v>
+      </c>
+      <c r="C39" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D39" s="95">
+        <f>F12*C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="96">
+        <f>F7*MAX(0,(F10-(17-1))/F10)+F8*MIN(17,F10)</f>
+        <v/>
+      </c>
+      <c r="F39" s="97">
+        <f>E39*F18</f>
+        <v/>
+      </c>
+      <c r="G39" s="94">
+        <f>E39/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H39" s="94">
+        <f>F13+F16+F17*F39</f>
+        <v/>
+      </c>
+      <c r="I39" s="98">
+        <f>F39-D39-G39-H39</f>
+        <v/>
+      </c>
+      <c r="J39" s="99">
+        <f>J38+I39</f>
+        <v/>
+      </c>
+      <c r="K39" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="B40" s="93" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="94">
+        <f>F8*F9</f>
+        <v/>
+      </c>
+      <c r="D40" s="95">
+        <f>F12*C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="96">
+        <f>F7*MAX(0,(F10-(18-1))/F10)+F8*MIN(18,F10)</f>
+        <v/>
+      </c>
+      <c r="F40" s="97">
+        <f>E40*F18</f>
+        <v/>
+      </c>
+      <c r="G40" s="94">
+        <f>E40/F14*F15/12</f>
+        <v/>
+      </c>
+      <c r="H40" s="94">
+        <f>F13+F16+F17*F40</f>
+        <v/>
+      </c>
+      <c r="I40" s="98">
+        <f>F40-D40-G40-H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="99">
+        <f>J39+I40</f>
+        <v/>
+      </c>
+      <c r="K40" s="100">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cash-flow trough (min cumulative)</t>
+        </is>
+      </c>
+      <c r="F42" s="102">
+        <f>MIN(J23:J40)</f>
+        <v/>
+      </c>
+      <c r="G42" s="103" t="inlineStr">
+        <is>
+          <t>lowest your cash gets during the ramp</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Month-1 cash vs run-rate profit gap</t>
+        </is>
+      </c>
+      <c r="F43" s="102">
+        <f>K23-F23</f>
+        <v/>
+      </c>
+      <c r="G43" s="103" t="inlineStr">
+        <is>
+          <t>collections shortfall vs steady-state in month 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="104">
+        <f>IF(MIN(J23:J40)&lt;0,"CASH GOES NEGATIVE DURING RAMP — secure a buffer / line of credit before scaling intake","CASH STAYS POSITIVE — but early months bank well below run-rate; keep the buffer intact")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46"/>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B21:K21"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B45:K46"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B10:E10"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I23:I40">
+    <cfRule type="expression" priority="1" dxfId="7">
+      <formula>I23&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J23:J40">
+    <cfRule type="expression" priority="2" dxfId="7">
+      <formula>J23&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B45">
+    <cfRule type="expression" priority="3" dxfId="8">
+      <formula>MIN(J23:J40)&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="9">
+      <formula>MIN(J23:J40)&gt;=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B2A4A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="105" t="inlineStr">
+        <is>
+          <t>COMP OPTIMIZER  ·  Highest James Rate the Firm Can Afford</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="66" t="inlineStr">
+        <is>
+          <t>Solves for the maximum James commission % that still (a) keeps the firm no worse than the old model, and (b) holds a target net margin. All else linked from Profitability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Target net margin (floor)</t>
+        </is>
+      </c>
+      <c r="C6" s="107" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D6" s="108" t="inlineStr">
+        <is>
+          <t>current James commission % →</t>
+        </is>
+      </c>
+      <c r="E6" s="109">
+        <f>'Profitability'!E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RESULTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Firm net profit — OLD model</t>
+        </is>
+      </c>
+      <c r="C9" s="94">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+      <c r="D9" s="103" t="inlineStr">
+        <is>
+          <t>the floor to beat</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Firm net profit — NEW (at current James %)</t>
+        </is>
+      </c>
+      <c r="C10" s="94">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-'Profitability'!E14*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D10" s="103" t="inlineStr">
+        <is>
+          <t>with James commission applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max James % — stay ACCRETIVE vs old</t>
+        </is>
+      </c>
+      <c r="C11" s="110">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))))/('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D11" s="103" t="inlineStr">
+        <is>
+          <t>above this, firm earns less than old model</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Max James % — hold target margin</t>
+        </is>
+      </c>
+      <c r="C12" s="110">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-C6*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9))/('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D12" s="103" t="inlineStr">
+        <is>
+          <t>above this, margin falls below the floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Headroom on James % (accretive − current)</t>
+        </is>
+      </c>
+      <c r="C13" s="111">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))))/('Profitability'!E11*52*'Profitability'!E6)-'Profitability'!E14</f>
+        <v/>
+      </c>
+      <c r="D13" s="103" t="inlineStr">
+        <is>
+          <t>how much room to raise his rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SENSITIVITY — James commission % vs firm profit &amp; his pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="B16" s="113" t="inlineStr">
+        <is>
+          <t>James comm %</t>
+        </is>
+      </c>
+      <c r="C16" s="113" t="inlineStr">
+        <is>
+          <t>James pay ($)</t>
+        </is>
+      </c>
+      <c r="D16" s="113" t="inlineStr">
+        <is>
+          <t>Firm net profit</t>
+        </is>
+      </c>
+      <c r="E16" s="113" t="inlineStr">
+        <is>
+          <t>Net margin</t>
+        </is>
+      </c>
+      <c r="F16" s="113" t="inlineStr">
+        <is>
+          <t>Beats old?</t>
+        </is>
+      </c>
+      <c r="G16" s="114" t="inlineStr">
+        <is>
+          <t>Old-model net</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="115" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="116">
+        <f>'Profitability'!E13+B17*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D17" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E17" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F17" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G17" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="115" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C18" s="116">
+        <f>'Profitability'!E13+B18*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D18" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E18" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F18" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G18" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="B19" s="115" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C19" s="116">
+        <f>'Profitability'!E13+B19*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D19" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E19" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F19" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G19" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="B20" s="115" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C20" s="116">
+        <f>'Profitability'!E13+B20*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D20" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E20" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F20" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G20" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="115" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C21" s="116">
+        <f>'Profitability'!E13+B21*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D21" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E21" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F21" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G21" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="115" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C22" s="116">
+        <f>'Profitability'!E13+B22*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D22" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E22" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F22" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G22" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="115" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C23" s="116">
+        <f>'Profitability'!E13+B23*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D23" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E23" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F23" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G23" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="115" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="C24" s="116">
+        <f>'Profitability'!E13+B24*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D24" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E24" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F24" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G24" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="115" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C25" s="116">
+        <f>'Profitability'!E13+B25*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D25" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E25" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F25" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G25" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="115" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="C26" s="116">
+        <f>'Profitability'!E13+B26*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D26" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E26" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F26" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G26" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="B27" s="115" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C27" s="116">
+        <f>'Profitability'!E13+B27*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D27" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E27" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F27" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G27" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="B28" s="115" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="C28" s="116">
+        <f>'Profitability'!E13+B28*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D28" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E28" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F28" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G28" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="B29" s="115" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C29" s="116">
+        <f>'Profitability'!E13+B29*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="D29" s="98">
+        <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6)</f>
+        <v/>
+      </c>
+      <c r="E29" s="117">
+        <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
+        <v/>
+      </c>
+      <c r="F29" s="93">
+        <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
+        <v/>
+      </c>
+      <c r="G29" s="100">
+        <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="D10:F10"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F17:F29">
+    <cfRule type="expression" priority="1" dxfId="10">
+      <formula>F17="yes"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="11">
+      <formula>F17="no"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E29">
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>E17&lt;C6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile capacity vs David's actual case-handling estimate
Capacity Lite: add David's operational cases-per-manager estimate (80-100,
default 90) as a first-class input, shown side-by-side against the
revenue-derived figure (143). Model now uses the BINDING (lower) number
so capacity, utilization, verdict and the 12-month projection reflect
reality. Flag fires when the base price can't reach the $1M/mgr target
at David's caseload, showing the shortfall and the price (or headcount)
needed to close it. With David's 90, utilization reads ~86% (ADD
CAPACITY) vs the old ~54% (SELL MORE).

Propagate: Profitability/Cash Timing/Comp Optimizer now size the
case-manager team off David's binding cases/mgr, so required headcount
and cost reflect his real numbers across every tab.
</commit_message>
<xml_diff>
--- a/Capacity-Lite.xlsx
+++ b/Capacity-Lite.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -201,6 +201,24 @@
       <color rgb="00FFFFFF"/>
       <sz val="18"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007A8499"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="009C7415"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B3402E"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -369,7 +387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -704,11 +722,131 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="33" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
     <dxf>
       <font>
         <b val="1"/>
@@ -831,6 +969,20 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4D8D1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9ECE2"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -916,7 +1068,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Active book value vs. comfortable revenue capacity</a:t>
+              <a:t>Active book value vs David's comfortable capacity</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -930,11 +1082,11 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Capacity Lite'!G38</f>
+              <f>'Capacity Lite'!G51</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln w="30000">
               <a:solidFill>
                 <a:srgbClr val="C8961E"/>
               </a:solidFill>
@@ -951,12 +1103,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Capacity Lite'!$B$39:$B$51</f>
+              <f>'Capacity Lite'!$B$52:$B$64</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capacity Lite'!$G$39:$G$51</f>
+              <f>'Capacity Lite'!$G$52:$G$64</f>
             </numRef>
           </val>
         </ser>
@@ -965,7 +1117,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Capacity Lite'!J38</f>
+              <f>'Capacity Lite'!J51</f>
             </strRef>
           </tx>
           <spPr>
@@ -986,12 +1138,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Capacity Lite'!$B$39:$B$51</f>
+              <f>'Capacity Lite'!$B$52:$B$64</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capacity Lite'!$J$39:$J$51</f>
+              <f>'Capacity Lite'!$J$52:$J$64</f>
             </numRef>
           </val>
         </ser>
@@ -1016,21 +1168,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Active book value</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -2051,1152 +2188,1208 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J61"/>
+  <dimension ref="B2:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="2" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="37" t="inlineStr">
-        <is>
-          <t>CAPACITY LITE  ·  Tax Resolution  ·  Revenue-Based (v2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="B3" s="38" t="inlineStr">
-        <is>
-          <t>Capacity is a REVENUE ceiling per case manager; case counts are derived. Edit the yellow (team/data) and blue (David's model definitions) cells.  Model owner: David.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="39" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="118" t="inlineStr">
+        <is>
+          <t>CAPACITY LITE  ·  Revenue-Based  ·  Calculated vs David's Actuals</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="66" t="inlineStr">
+        <is>
+          <t>Capacity is a revenue ceiling per manager, but it can't exceed how many cases a manager can actually carry. The model uses the BINDING (lower) of the two and flags when the base price can't reach the revenue target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="119" t="inlineStr">
         <is>
           <t xml:space="preserve">  INPUTS</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="B6" s="57" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Full-capacity case managers (FTE)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="121" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>people   —   Ramped case managers at full capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="B7" s="57" t="inlineStr">
+      <c r="G6" s="122" t="inlineStr">
+        <is>
+          <t>Ramped managers at full capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case managers in training (count)</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="123" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>people   —   Each counts as 0.5 FTE until ramped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="B8" s="57" t="inlineStr">
+      <c r="G7" s="122" t="inlineStr">
+        <is>
+          <t>Each counts as 0.5 FTE until ramped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Current active (open) cases</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="123" t="n">
         <v>350</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>cases   —   Your open book right now, all managers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="B9" s="57" t="inlineStr">
+      <c r="G8" s="122" t="inlineStr">
+        <is>
+          <t>Open book right now, all managers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  New cases signed / week</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="123" t="n">
         <v>25</v>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>cases/wk   —   Sales goal: 3 reps + James @ 6 follow-ups/day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue capacity per manager ($/yr)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
+      <c r="G9" s="122" t="inlineStr">
+        <is>
+          <t>Sales goal: 3 reps + James.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Revenue capacity per manager ($/yr)  — TARGET</t>
+        </is>
+      </c>
+      <c r="E10" s="124" t="n">
         <v>1000000</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>per mgr   —   David: 'full capacity' = ~$1M active book.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="57" t="inlineStr">
+      <c r="G10" s="122" t="inlineStr">
+        <is>
+          <t>David's aspirational 'full capacity'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case value ($)</t>
         </is>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="124" t="n">
         <v>7000</v>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>per case   —   David.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="57" t="inlineStr">
+      <c r="G11" s="122" t="inlineStr">
+        <is>
+          <t>David — the base price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  David's est. cases per manager (operational)</t>
+        </is>
+      </c>
+      <c r="E12" s="125" t="n">
+        <v>90</v>
+      </c>
+      <c r="G12" s="122" t="inlineStr">
+        <is>
+          <t>David's REAL estimate: 80–100. Caps the calc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case lifespan (months)</t>
         </is>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E13" s="126" t="n">
         <v>12</v>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>months   —   David's estimate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="57" t="inlineStr">
+      <c r="G13" s="122" t="inlineStr">
+        <is>
+          <t>David's estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Comfort ceiling (% of capacity)</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E14" s="127" t="n">
         <v>0.85</v>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>of cap   —   Utilization you don't want to exceed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  DERIVED CAPACITY</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="40" t="inlineStr">
+      <c r="G14" s="122" t="inlineStr">
+        <is>
+          <t>Utilization you don't want to exceed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CAPACITY:  CALCULATED  vs  DAVID'S ACTUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="129" t="inlineStr"/>
+      <c r="E17" s="130" t="inlineStr">
+        <is>
+          <t>CALCULATED (rev-derived)</t>
+        </is>
+      </c>
+      <c r="G17" s="131" t="inlineStr">
+        <is>
+          <t>DAVID'S ACTUAL (operational)</t>
+        </is>
+      </c>
+      <c r="H17" s="132" t="inlineStr">
+        <is>
+          <t>← the column that reflects reality</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cases per manager</t>
+        </is>
+      </c>
+      <c r="E18" s="133">
+        <f>E10/E11</f>
+        <v/>
+      </c>
+      <c r="G18" s="134">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="H18" s="135" t="inlineStr">
+        <is>
+          <t>$1M÷$7k = 143   vs   David ~90</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Revenue per manager</t>
+        </is>
+      </c>
+      <c r="E19" s="136">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="G19" s="137">
+        <f>E12*E11</f>
+        <v/>
+      </c>
+      <c r="H19" s="135" t="inlineStr">
+        <is>
+          <t>David: 90 × $7k = $630k, not $1M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Effective case managers (FTE)</t>
         </is>
       </c>
-      <c r="E15" s="13">
+      <c r="E20" s="138">
         <f>E6+0.5*E7</f>
         <v/>
       </c>
-      <c r="F15" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   full + ½ × trainees</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Max active cases per manager</t>
-        </is>
-      </c>
-      <c r="E16" s="13">
-        <f>E10/E11</f>
-        <v/>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   revenue ceiling ÷ case value  (≈143)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Total revenue capacity</t>
-        </is>
-      </c>
-      <c r="E17" s="15">
-        <f>E15*E10</f>
-        <v/>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   effective FTE × ceiling/mgr</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Total case capacity</t>
-        </is>
-      </c>
-      <c r="E18" s="13">
-        <f>E15*E16</f>
-        <v/>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   derived case ceiling</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Comfortable revenue capacity</t>
-        </is>
-      </c>
-      <c r="E19" s="15">
-        <f>E17*E13</f>
-        <v/>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   total capacity × comfort ceiling</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Historical benchmark (cases/mgr, w/ admin)</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="n">
-        <v>130</v>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   prior reference — compare to ~143 above</t>
+      <c r="G20" s="135" t="inlineStr">
+        <is>
+          <t>full + ½ × trainees</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CURRENT STATE</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B21" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total case capacity (× FTE)</t>
+        </is>
+      </c>
+      <c r="E21" s="133">
+        <f>E20*E18</f>
+        <v/>
+      </c>
+      <c r="G21" s="134">
+        <f>E20*G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total revenue capacity (× FTE)</t>
+        </is>
+      </c>
+      <c r="E22" s="136">
+        <f>E20*E19</f>
+        <v/>
+      </c>
+      <c r="G22" s="137">
+        <f>E20*G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ► Effective (binding) cases per manager</t>
+        </is>
+      </c>
+      <c r="E23" s="140">
+        <f>MIN(E18,G18)</f>
+        <v/>
+      </c>
+      <c r="G23" s="141" t="inlineStr">
+        <is>
+          <t>the LOWER of the two — drives the whole model &amp; other tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total revenue shortfall vs target</t>
+        </is>
+      </c>
+      <c r="E24" s="142">
+        <f>G22-E22</f>
+        <v/>
+      </c>
+      <c r="G24" s="132" t="inlineStr">
+        <is>
+          <t>David's total capacity minus the calculated target</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case value needed to hit $1M at David's caseload</t>
+        </is>
+      </c>
+      <c r="E25" s="143">
+        <f>E10/E12</f>
+        <v/>
+      </c>
+      <c r="G25" s="132" t="inlineStr">
+        <is>
+          <t>raise price to here, or accept the lower ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Model total revenue capacity (binding)</t>
+        </is>
+      </c>
+      <c r="E27" s="137">
+        <f>E20*E23*E11</f>
+        <v/>
+      </c>
+      <c r="G27" s="135" t="inlineStr">
+        <is>
+          <t>effective FTE × binding cases/mgr × case value</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Model comfortable capacity (at ceiling)</t>
+        </is>
+      </c>
+      <c r="E28" s="137">
+        <f>E27*E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CAPACITY / PRICE FLAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="145">
+        <f>IF(G18&lt;E18,"⚠ CAN'T HIT $1M/MGR AT BASE PRICE — At David's "&amp;TEXT(G18,"0")&amp;" cases/mgr each manager tops out at "&amp;TEXT(G19,"$#,##0")&amp;"/yr. "&amp;TEXT(E20,"0.0")&amp;" FTE = "&amp;TEXT(G22,"$#,##0")&amp;" capacity vs the "&amp;TEXT(E22,"$#,##0")&amp;" target ("&amp;TEXT(E24,"$#,##0")&amp;" short). Fix: raise price to "&amp;TEXT(E25,"$#,##0")&amp;"/case, or add managers, or lower the target.","✓ David's operational capacity supports the revenue target at the current base price.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1"/>
+    <row r="33" ht="22" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CURRENT STATE  (against David's binding capacity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Current active book value</t>
         </is>
       </c>
-      <c r="E22" s="15">
+      <c r="E36" s="146">
         <f>E8*E11</f>
         <v/>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="G36" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   open cases × case value</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="40" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue utilization</t>
         </is>
       </c>
-      <c r="E23" s="17">
-        <f>E22/E17</f>
-        <v/>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   book value ÷ total revenue capacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="40" t="inlineStr">
+      <c r="E37" s="147">
+        <f>E36/E27</f>
+        <v/>
+      </c>
+      <c r="G37" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   book value ÷ binding revenue capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Headroom to comfort ($)</t>
         </is>
       </c>
-      <c r="E24" s="15">
-        <f>E19-E22</f>
-        <v/>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="E38" s="146">
+        <f>E28-E36</f>
+        <v/>
+      </c>
+      <c r="G38" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   room before the comfort ceiling</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="40" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Headroom to comfort (cases)</t>
         </is>
       </c>
-      <c r="E25" s="13">
-        <f>E24/E11</f>
-        <v/>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   same headroom expressed in cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="40" t="inlineStr">
+      <c r="E39" s="148">
+        <f>E38/E11</f>
+        <v/>
+      </c>
+      <c r="G39" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   same headroom in cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  New cases / month</t>
         </is>
       </c>
-      <c r="E26" s="13">
+      <c r="E40" s="148">
         <f>E9*52/12</f>
         <v/>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="G40" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   25/wk ≈ 108/mo</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="40" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cases closing / month</t>
         </is>
       </c>
-      <c r="E27" s="13">
-        <f>E8/E12</f>
-        <v/>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="E41" s="148">
+        <f>E8/E13</f>
+        <v/>
+      </c>
+      <c r="G41" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   ≈ open ÷ lifespan</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="40" t="inlineStr">
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Net case growth / month</t>
         </is>
       </c>
-      <c r="E28" s="13">
-        <f>E26-E27</f>
-        <v/>
-      </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="E42" s="148">
+        <f>E40-E41</f>
+        <v/>
+      </c>
+      <c r="G42" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   new − closing</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Net revenue growth / month</t>
-        </is>
-      </c>
-      <c r="E29" s="15">
-        <f>E28*E11</f>
-        <v/>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   net case growth × case value</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="40" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Months to comfortably full</t>
         </is>
       </c>
-      <c r="E30" s="13">
-        <f>IF(E28&lt;=0,"stable / shrinking",IF(E25&lt;=0,"already over",E25/E28))</f>
-        <v/>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="E43" s="148">
+        <f>IF(E42&lt;=0,"stable / shrinking",IF(E38&lt;=0,"already over",E38/E42))</f>
+        <v/>
+      </c>
+      <c r="G43" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">   headroom ÷ net growth</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Implied annual revenue throughput</t>
-        </is>
-      </c>
-      <c r="E31" s="15">
-        <f>E22*(12/E12)</f>
-        <v/>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   = book value when lifespan = 12 mo</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="18">
-        <f>IF(E23&gt;=E13,"ADD CAPACITY",IF(E23&lt;=E13-0.2,"SELL MORE","MAINTAIN"))</f>
-        <v/>
-      </c>
-      <c r="C33" s="30" t="n"/>
-      <c r="D33" s="30" t="n"/>
-      <c r="E33" s="30" t="n"/>
-      <c r="F33" s="30" t="n"/>
-      <c r="G33" s="30" t="n"/>
-      <c r="H33" s="30" t="n"/>
-      <c r="I33" s="30" t="n"/>
-      <c r="J33" s="31" t="n"/>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="B34" s="32" t="n"/>
-      <c r="J34" s="33" t="n"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="34" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="35" t="n"/>
-      <c r="E35" s="35" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="35" t="n"/>
-      <c r="H35" s="35" t="n"/>
-      <c r="I35" s="35" t="n"/>
-      <c r="J35" s="36" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Three states: at/above the comfort ceiling → ADD CAPACITY · more than 20 pts below → SELL MORE · in between → MAINTAIN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  12-MONTH PROJECTION  (assumes intake, case value &amp; lifespan hold steady)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="20" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="18">
+        <f>IF(E37&gt;=E14,"ADD CAPACITY",IF(E37&lt;=E14-0.2,"SELL MORE","MAINTAIN"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48">
+      <c r="B48" s="149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Now measured against David's real capacity — expect a tighter read than the old $1M-based number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="B50" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  12-MONTH PROJECTION  (utilization vs David's binding capacity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C38" s="20" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Open (start)</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="F38" s="20" t="inlineStr">
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>Open (end)</t>
         </is>
       </c>
-      <c r="G38" s="20" t="inlineStr">
+      <c r="G51" s="20" t="inlineStr">
         <is>
           <t>Book value</t>
         </is>
       </c>
-      <c r="H38" s="20" t="inlineStr">
+      <c r="H51" s="20" t="inlineStr">
         <is>
           <t>Rev. util.</t>
         </is>
       </c>
-      <c r="I38" s="20" t="inlineStr">
+      <c r="I51" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J38" s="20" t="inlineStr">
+      <c r="J51" s="20" t="inlineStr">
         <is>
           <t>Comfort cap ($)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="21" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="150" t="inlineStr">
         <is>
           <t>Now</t>
         </is>
       </c>
-      <c r="C39" s="22" t="inlineStr">
+      <c r="C52" s="151" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D52" s="151" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E52" s="151" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F39" s="23">
+      <c r="F52" s="152">
         <f>E8</f>
         <v/>
       </c>
-      <c r="G39" s="56">
-        <f>F39*$E$11</f>
-        <v/>
-      </c>
-      <c r="H39" s="25">
-        <f>G39/$E$17</f>
-        <v/>
-      </c>
-      <c r="I39" s="26">
-        <f>IF(H39&gt;=$E$13,"Add capacity",IF(H39&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J39" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="26" t="inlineStr">
+      <c r="G52" s="153">
+        <f>F52*$E$11</f>
+        <v/>
+      </c>
+      <c r="H52" s="154">
+        <f>G52/$E$27</f>
+        <v/>
+      </c>
+      <c r="I52" s="155">
+        <f>IF(H52&gt;=$E$14,"Add capacity",IF(H52&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J52" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="155" t="inlineStr">
         <is>
           <t>Mo 1</t>
         </is>
       </c>
-      <c r="C40" s="55">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="D40" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E40" s="55">
-        <f>C40/$E$12</f>
-        <v/>
-      </c>
-      <c r="F40" s="23">
-        <f>MAX(0,C40+D40-E40)</f>
-        <v/>
-      </c>
-      <c r="G40" s="56">
-        <f>F40*$E$11</f>
-        <v/>
-      </c>
-      <c r="H40" s="25">
-        <f>G40/$E$17</f>
-        <v/>
-      </c>
-      <c r="I40" s="26">
-        <f>IF(H40&gt;=$E$13,"Add capacity",IF(H40&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J40" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="26" t="inlineStr">
+      <c r="C53" s="157">
+        <f>F52</f>
+        <v/>
+      </c>
+      <c r="D53" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E53" s="157">
+        <f>C53/$E$13</f>
+        <v/>
+      </c>
+      <c r="F53" s="152">
+        <f>MAX(0,C53+D53-E53)</f>
+        <v/>
+      </c>
+      <c r="G53" s="153">
+        <f>F53*$E$11</f>
+        <v/>
+      </c>
+      <c r="H53" s="154">
+        <f>G53/$E$27</f>
+        <v/>
+      </c>
+      <c r="I53" s="155">
+        <f>IF(H53&gt;=$E$14,"Add capacity",IF(H53&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J53" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="155" t="inlineStr">
         <is>
           <t>Mo 2</t>
         </is>
       </c>
-      <c r="C41" s="55">
-        <f>F40</f>
-        <v/>
-      </c>
-      <c r="D41" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E41" s="55">
-        <f>C41/$E$12</f>
-        <v/>
-      </c>
-      <c r="F41" s="23">
-        <f>MAX(0,C41+D41-E41)</f>
-        <v/>
-      </c>
-      <c r="G41" s="56">
-        <f>F41*$E$11</f>
-        <v/>
-      </c>
-      <c r="H41" s="25">
-        <f>G41/$E$17</f>
-        <v/>
-      </c>
-      <c r="I41" s="26">
-        <f>IF(H41&gt;=$E$13,"Add capacity",IF(H41&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J41" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="26" t="inlineStr">
+      <c r="C54" s="157">
+        <f>F53</f>
+        <v/>
+      </c>
+      <c r="D54" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E54" s="157">
+        <f>C54/$E$13</f>
+        <v/>
+      </c>
+      <c r="F54" s="152">
+        <f>MAX(0,C54+D54-E54)</f>
+        <v/>
+      </c>
+      <c r="G54" s="153">
+        <f>F54*$E$11</f>
+        <v/>
+      </c>
+      <c r="H54" s="154">
+        <f>G54/$E$27</f>
+        <v/>
+      </c>
+      <c r="I54" s="155">
+        <f>IF(H54&gt;=$E$14,"Add capacity",IF(H54&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J54" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="155" t="inlineStr">
         <is>
           <t>Mo 3</t>
         </is>
       </c>
-      <c r="C42" s="55">
-        <f>F41</f>
-        <v/>
-      </c>
-      <c r="D42" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E42" s="55">
-        <f>C42/$E$12</f>
-        <v/>
-      </c>
-      <c r="F42" s="23">
-        <f>MAX(0,C42+D42-E42)</f>
-        <v/>
-      </c>
-      <c r="G42" s="56">
-        <f>F42*$E$11</f>
-        <v/>
-      </c>
-      <c r="H42" s="25">
-        <f>G42/$E$17</f>
-        <v/>
-      </c>
-      <c r="I42" s="26">
-        <f>IF(H42&gt;=$E$13,"Add capacity",IF(H42&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J42" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="26" t="inlineStr">
+      <c r="C55" s="157">
+        <f>F54</f>
+        <v/>
+      </c>
+      <c r="D55" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E55" s="157">
+        <f>C55/$E$13</f>
+        <v/>
+      </c>
+      <c r="F55" s="152">
+        <f>MAX(0,C55+D55-E55)</f>
+        <v/>
+      </c>
+      <c r="G55" s="153">
+        <f>F55*$E$11</f>
+        <v/>
+      </c>
+      <c r="H55" s="154">
+        <f>G55/$E$27</f>
+        <v/>
+      </c>
+      <c r="I55" s="155">
+        <f>IF(H55&gt;=$E$14,"Add capacity",IF(H55&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J55" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="155" t="inlineStr">
         <is>
           <t>Mo 4</t>
         </is>
       </c>
-      <c r="C43" s="55">
-        <f>F42</f>
-        <v/>
-      </c>
-      <c r="D43" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E43" s="55">
-        <f>C43/$E$12</f>
-        <v/>
-      </c>
-      <c r="F43" s="23">
-        <f>MAX(0,C43+D43-E43)</f>
-        <v/>
-      </c>
-      <c r="G43" s="56">
-        <f>F43*$E$11</f>
-        <v/>
-      </c>
-      <c r="H43" s="25">
-        <f>G43/$E$17</f>
-        <v/>
-      </c>
-      <c r="I43" s="26">
-        <f>IF(H43&gt;=$E$13,"Add capacity",IF(H43&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J43" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="26" t="inlineStr">
+      <c r="C56" s="157">
+        <f>F55</f>
+        <v/>
+      </c>
+      <c r="D56" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E56" s="157">
+        <f>C56/$E$13</f>
+        <v/>
+      </c>
+      <c r="F56" s="152">
+        <f>MAX(0,C56+D56-E56)</f>
+        <v/>
+      </c>
+      <c r="G56" s="153">
+        <f>F56*$E$11</f>
+        <v/>
+      </c>
+      <c r="H56" s="154">
+        <f>G56/$E$27</f>
+        <v/>
+      </c>
+      <c r="I56" s="155">
+        <f>IF(H56&gt;=$E$14,"Add capacity",IF(H56&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J56" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="155" t="inlineStr">
         <is>
           <t>Mo 5</t>
         </is>
       </c>
-      <c r="C44" s="55">
-        <f>F43</f>
-        <v/>
-      </c>
-      <c r="D44" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E44" s="55">
-        <f>C44/$E$12</f>
-        <v/>
-      </c>
-      <c r="F44" s="23">
-        <f>MAX(0,C44+D44-E44)</f>
-        <v/>
-      </c>
-      <c r="G44" s="56">
-        <f>F44*$E$11</f>
-        <v/>
-      </c>
-      <c r="H44" s="25">
-        <f>G44/$E$17</f>
-        <v/>
-      </c>
-      <c r="I44" s="26">
-        <f>IF(H44&gt;=$E$13,"Add capacity",IF(H44&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J44" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="26" t="inlineStr">
+      <c r="C57" s="157">
+        <f>F56</f>
+        <v/>
+      </c>
+      <c r="D57" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E57" s="157">
+        <f>C57/$E$13</f>
+        <v/>
+      </c>
+      <c r="F57" s="152">
+        <f>MAX(0,C57+D57-E57)</f>
+        <v/>
+      </c>
+      <c r="G57" s="153">
+        <f>F57*$E$11</f>
+        <v/>
+      </c>
+      <c r="H57" s="154">
+        <f>G57/$E$27</f>
+        <v/>
+      </c>
+      <c r="I57" s="155">
+        <f>IF(H57&gt;=$E$14,"Add capacity",IF(H57&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J57" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="155" t="inlineStr">
         <is>
           <t>Mo 6</t>
         </is>
       </c>
-      <c r="C45" s="55">
-        <f>F44</f>
-        <v/>
-      </c>
-      <c r="D45" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E45" s="55">
-        <f>C45/$E$12</f>
-        <v/>
-      </c>
-      <c r="F45" s="23">
-        <f>MAX(0,C45+D45-E45)</f>
-        <v/>
-      </c>
-      <c r="G45" s="56">
-        <f>F45*$E$11</f>
-        <v/>
-      </c>
-      <c r="H45" s="25">
-        <f>G45/$E$17</f>
-        <v/>
-      </c>
-      <c r="I45" s="26">
-        <f>IF(H45&gt;=$E$13,"Add capacity",IF(H45&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J45" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="26" t="inlineStr">
+      <c r="C58" s="157">
+        <f>F57</f>
+        <v/>
+      </c>
+      <c r="D58" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E58" s="157">
+        <f>C58/$E$13</f>
+        <v/>
+      </c>
+      <c r="F58" s="152">
+        <f>MAX(0,C58+D58-E58)</f>
+        <v/>
+      </c>
+      <c r="G58" s="153">
+        <f>F58*$E$11</f>
+        <v/>
+      </c>
+      <c r="H58" s="154">
+        <f>G58/$E$27</f>
+        <v/>
+      </c>
+      <c r="I58" s="155">
+        <f>IF(H58&gt;=$E$14,"Add capacity",IF(H58&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J58" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="155" t="inlineStr">
         <is>
           <t>Mo 7</t>
         </is>
       </c>
-      <c r="C46" s="55">
-        <f>F45</f>
-        <v/>
-      </c>
-      <c r="D46" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E46" s="55">
-        <f>C46/$E$12</f>
-        <v/>
-      </c>
-      <c r="F46" s="23">
-        <f>MAX(0,C46+D46-E46)</f>
-        <v/>
-      </c>
-      <c r="G46" s="56">
-        <f>F46*$E$11</f>
-        <v/>
-      </c>
-      <c r="H46" s="25">
-        <f>G46/$E$17</f>
-        <v/>
-      </c>
-      <c r="I46" s="26">
-        <f>IF(H46&gt;=$E$13,"Add capacity",IF(H46&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J46" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="26" t="inlineStr">
+      <c r="C59" s="157">
+        <f>F58</f>
+        <v/>
+      </c>
+      <c r="D59" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E59" s="157">
+        <f>C59/$E$13</f>
+        <v/>
+      </c>
+      <c r="F59" s="152">
+        <f>MAX(0,C59+D59-E59)</f>
+        <v/>
+      </c>
+      <c r="G59" s="153">
+        <f>F59*$E$11</f>
+        <v/>
+      </c>
+      <c r="H59" s="154">
+        <f>G59/$E$27</f>
+        <v/>
+      </c>
+      <c r="I59" s="155">
+        <f>IF(H59&gt;=$E$14,"Add capacity",IF(H59&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J59" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="155" t="inlineStr">
         <is>
           <t>Mo 8</t>
         </is>
       </c>
-      <c r="C47" s="55">
-        <f>F46</f>
-        <v/>
-      </c>
-      <c r="D47" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E47" s="55">
-        <f>C47/$E$12</f>
-        <v/>
-      </c>
-      <c r="F47" s="23">
-        <f>MAX(0,C47+D47-E47)</f>
-        <v/>
-      </c>
-      <c r="G47" s="56">
-        <f>F47*$E$11</f>
-        <v/>
-      </c>
-      <c r="H47" s="25">
-        <f>G47/$E$17</f>
-        <v/>
-      </c>
-      <c r="I47" s="26">
-        <f>IF(H47&gt;=$E$13,"Add capacity",IF(H47&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J47" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="26" t="inlineStr">
+      <c r="C60" s="157">
+        <f>F59</f>
+        <v/>
+      </c>
+      <c r="D60" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E60" s="157">
+        <f>C60/$E$13</f>
+        <v/>
+      </c>
+      <c r="F60" s="152">
+        <f>MAX(0,C60+D60-E60)</f>
+        <v/>
+      </c>
+      <c r="G60" s="153">
+        <f>F60*$E$11</f>
+        <v/>
+      </c>
+      <c r="H60" s="154">
+        <f>G60/$E$27</f>
+        <v/>
+      </c>
+      <c r="I60" s="155">
+        <f>IF(H60&gt;=$E$14,"Add capacity",IF(H60&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J60" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="155" t="inlineStr">
         <is>
           <t>Mo 9</t>
         </is>
       </c>
-      <c r="C48" s="55">
-        <f>F47</f>
-        <v/>
-      </c>
-      <c r="D48" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E48" s="55">
-        <f>C48/$E$12</f>
-        <v/>
-      </c>
-      <c r="F48" s="23">
-        <f>MAX(0,C48+D48-E48)</f>
-        <v/>
-      </c>
-      <c r="G48" s="56">
-        <f>F48*$E$11</f>
-        <v/>
-      </c>
-      <c r="H48" s="25">
-        <f>G48/$E$17</f>
-        <v/>
-      </c>
-      <c r="I48" s="26">
-        <f>IF(H48&gt;=$E$13,"Add capacity",IF(H48&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J48" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="26" t="inlineStr">
+      <c r="C61" s="157">
+        <f>F60</f>
+        <v/>
+      </c>
+      <c r="D61" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E61" s="157">
+        <f>C61/$E$13</f>
+        <v/>
+      </c>
+      <c r="F61" s="152">
+        <f>MAX(0,C61+D61-E61)</f>
+        <v/>
+      </c>
+      <c r="G61" s="153">
+        <f>F61*$E$11</f>
+        <v/>
+      </c>
+      <c r="H61" s="154">
+        <f>G61/$E$27</f>
+        <v/>
+      </c>
+      <c r="I61" s="155">
+        <f>IF(H61&gt;=$E$14,"Add capacity",IF(H61&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J61" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="155" t="inlineStr">
         <is>
           <t>Mo 10</t>
         </is>
       </c>
-      <c r="C49" s="55">
-        <f>F48</f>
-        <v/>
-      </c>
-      <c r="D49" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E49" s="55">
-        <f>C49/$E$12</f>
-        <v/>
-      </c>
-      <c r="F49" s="23">
-        <f>MAX(0,C49+D49-E49)</f>
-        <v/>
-      </c>
-      <c r="G49" s="56">
-        <f>F49*$E$11</f>
-        <v/>
-      </c>
-      <c r="H49" s="25">
-        <f>G49/$E$17</f>
-        <v/>
-      </c>
-      <c r="I49" s="26">
-        <f>IF(H49&gt;=$E$13,"Add capacity",IF(H49&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J49" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="26" t="inlineStr">
+      <c r="C62" s="157">
+        <f>F61</f>
+        <v/>
+      </c>
+      <c r="D62" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E62" s="157">
+        <f>C62/$E$13</f>
+        <v/>
+      </c>
+      <c r="F62" s="152">
+        <f>MAX(0,C62+D62-E62)</f>
+        <v/>
+      </c>
+      <c r="G62" s="153">
+        <f>F62*$E$11</f>
+        <v/>
+      </c>
+      <c r="H62" s="154">
+        <f>G62/$E$27</f>
+        <v/>
+      </c>
+      <c r="I62" s="155">
+        <f>IF(H62&gt;=$E$14,"Add capacity",IF(H62&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J62" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="155" t="inlineStr">
         <is>
           <t>Mo 11</t>
         </is>
       </c>
-      <c r="C50" s="55">
-        <f>F49</f>
-        <v/>
-      </c>
-      <c r="D50" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E50" s="55">
-        <f>C50/$E$12</f>
-        <v/>
-      </c>
-      <c r="F50" s="23">
-        <f>MAX(0,C50+D50-E50)</f>
-        <v/>
-      </c>
-      <c r="G50" s="56">
-        <f>F50*$E$11</f>
-        <v/>
-      </c>
-      <c r="H50" s="25">
-        <f>G50/$E$17</f>
-        <v/>
-      </c>
-      <c r="I50" s="26">
-        <f>IF(H50&gt;=$E$13,"Add capacity",IF(H50&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J50" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="26" t="inlineStr">
+      <c r="C63" s="157">
+        <f>F62</f>
+        <v/>
+      </c>
+      <c r="D63" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E63" s="157">
+        <f>C63/$E$13</f>
+        <v/>
+      </c>
+      <c r="F63" s="152">
+        <f>MAX(0,C63+D63-E63)</f>
+        <v/>
+      </c>
+      <c r="G63" s="153">
+        <f>F63*$E$11</f>
+        <v/>
+      </c>
+      <c r="H63" s="154">
+        <f>G63/$E$27</f>
+        <v/>
+      </c>
+      <c r="I63" s="155">
+        <f>IF(H63&gt;=$E$14,"Add capacity",IF(H63&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J63" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="155" t="inlineStr">
         <is>
           <t>Mo 12</t>
         </is>
       </c>
-      <c r="C51" s="55">
-        <f>F50</f>
-        <v/>
-      </c>
-      <c r="D51" s="55">
-        <f>$E$26</f>
-        <v/>
-      </c>
-      <c r="E51" s="55">
-        <f>C51/$E$12</f>
-        <v/>
-      </c>
-      <c r="F51" s="23">
-        <f>MAX(0,C51+D51-E51)</f>
-        <v/>
-      </c>
-      <c r="G51" s="56">
-        <f>F51*$E$11</f>
-        <v/>
-      </c>
-      <c r="H51" s="25">
-        <f>G51/$E$17</f>
-        <v/>
-      </c>
-      <c r="I51" s="26">
-        <f>IF(H51&gt;=$E$13,"Add capacity",IF(H51&lt;=$E$13-0.2,"Sell more","Maintain"))</f>
-        <v/>
-      </c>
-      <c r="J51" s="27">
-        <f>$E$19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="51" t="inlineStr">
+      <c r="C64" s="157">
+        <f>F63</f>
+        <v/>
+      </c>
+      <c r="D64" s="157">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="E64" s="157">
+        <f>C64/$E$13</f>
+        <v/>
+      </c>
+      <c r="F64" s="152">
+        <f>MAX(0,C64+D64-E64)</f>
+        <v/>
+      </c>
+      <c r="G64" s="153">
+        <f>F64*$E$11</f>
+        <v/>
+      </c>
+      <c r="H64" s="154">
+        <f>G64/$E$27</f>
+        <v/>
+      </c>
+      <c r="I64" s="155">
+        <f>IF(H64&gt;=$E$14,"Add capacity",IF(H64&lt;=$E$14-0.2,"Sell more","Maintain"))</f>
+        <v/>
+      </c>
+      <c r="J64" s="156">
+        <f>$E$28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="B66" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="B54" s="29" t="inlineStr">
-        <is>
-          <t>•  Model: capacity is a revenue ceiling per case manager (David's definition); case counts are DERIVED from revenue ceiling ÷ average case value. David owns this model and its calculations going forward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="B55" s="29" t="inlineStr">
-        <is>
-          <t>•  $1M reconciliation: treated as ACTIVE BOOK VALUE at a point in time → max ≈143 cases/mgr. With a 12-month lifespan this equals annual revenue throughput (see that row). Historical 130/mgr was WITH admin support — shown as a benchmark. To adopt 130, lower the revenue ceiling (≈$910K) or raise case value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="B56" s="29" t="inlineStr">
-        <is>
-          <t>•  Trainees count as 0.5 FTE until ramped; adjust the trainee count as new hires gain experience.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="B57" s="29" t="inlineStr">
-        <is>
-          <t>•  New-case goal of 25/week (≈108/month) is the sales target supported by 3 reps + James at 6 follow-up calls/day — stress-test it here against staffing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="B58" s="29" t="inlineStr">
-        <is>
-          <t>•  Data hygiene: time logs are NOT yet reliable (sub-1-minute entries seen). Enforce a 15-minute minimum increment, tie compliance to compensation, before trusting any hours-based metric (full Atlas). This sheet is case/revenue-based and unaffected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="B59" s="29" t="inlineStr">
-        <is>
-          <t>•  Known reporting quirks — footnote, do not treat as signal: (1) one-day overlap between growth and sales reports from different date defaults; (2) date-selector bug can select two days at once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="30" customHeight="1">
-      <c r="B60" s="29" t="inlineStr">
-        <is>
-          <t>•  Inputs can be entered manually now or synced later via OAuth from the CRM / task manager — the input cells work either way.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="B61" s="29" t="inlineStr">
-        <is>
-          <t>•  The full Capacity Atlas (3 utilization tracks: case/hours/surge, projected hours, expected revenue, surge overflow, hiring/intake triggers, and a P&amp;L view) remains the aspirational map; this Lite sheet is the immediately usable version (per Vanessa — show David both).</t>
+    <row r="67" ht="30" customHeight="1">
+      <c r="B67" s="29" t="inlineStr">
+        <is>
+          <t>•  RECONCILIATION: '$1M per manager' implies ~143 cases at a $7,000 base price, but David estimates a manager realistically carries 80–100. The model now uses the BINDING (lower) figure — David's — so capacity, utilization and every downstream tab reflect reality, not the arithmetic ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="B68" s="29" t="inlineStr">
+        <is>
+          <t>•  The flag fires whenever David's operational cases/mgr is below the revenue-derived number: it means the base price can't reach the $1M target with that caseload. Options shown: raise price, add managers, or lower the target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="B69" s="29" t="inlineStr">
+        <is>
+          <t>•  Because capacity is now David's (~90 not ~143), utilization reads much higher than the old version — that is the point of your correction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="B70" s="29" t="inlineStr">
+        <is>
+          <t>•  Trainees = 0.5 FTE until ramped. Adjust as new hires gain experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="B71" s="29" t="inlineStr">
+        <is>
+          <t>•  The Profitability, Cash Timing and Comp Optimizer tabs now size the case-manager team off David's binding cases/mgr, so their headcount and cost reflect his real numbers too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="B72" s="29" t="inlineStr">
+        <is>
+          <t>•  All comp/cost figures on the other tabs remain placeholders pending David's actuals.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="B61:J61"/>
-    <mergeCell ref="B14:J14"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="B60:J60"/>
-    <mergeCell ref="F19:J19"/>
-    <mergeCell ref="F25:J25"/>
-    <mergeCell ref="B57:J57"/>
-    <mergeCell ref="B53:J53"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="F7:J7"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="F15:J15"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="F24:J24"/>
-    <mergeCell ref="F20:J20"/>
-    <mergeCell ref="F18:J18"/>
-    <mergeCell ref="B55:J55"/>
-    <mergeCell ref="F8:J8"/>
-    <mergeCell ref="F26:J26"/>
-    <mergeCell ref="F17:J17"/>
+  <mergeCells count="42">
+    <mergeCell ref="B67:J67"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="B69:J69"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="B68:J68"/>
     <mergeCell ref="B5:J5"/>
-    <mergeCell ref="B33:J35"/>
-    <mergeCell ref="F23:J23"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="F22:J22"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F27:J27"/>
-    <mergeCell ref="B54:J54"/>
-    <mergeCell ref="F9:J9"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="B45:J47"/>
+    <mergeCell ref="B50:J50"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="B72:J72"/>
     <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B59:J59"/>
-    <mergeCell ref="B56:J56"/>
-    <mergeCell ref="B58:J58"/>
-    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B66:J66"/>
+    <mergeCell ref="B31:J33"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="B71:J71"/>
+    <mergeCell ref="B70:J70"/>
     <mergeCell ref="B2:J2"/>
+    <mergeCell ref="G14:J14"/>
   </mergeCells>
-  <conditionalFormatting sqref="B33">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>ISNUMBER(SEARCH("ADD",B33))</formula>
+  <conditionalFormatting sqref="B31">
+    <cfRule type="expression" priority="1" dxfId="12">
+      <formula>G18&lt;E18</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>ISNUMBER(SEARCH("SELL",B33))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>ISNUMBER(SEARCH("MAINTAIN",B33))</formula>
+    <cfRule type="expression" priority="2" dxfId="13">
+      <formula>G18&gt;=E18</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H39:H51">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="B45">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>ISNUMBER(SEARCH("ADD",B45))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>ISNUMBER(SEARCH("SELL",B45))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>ISNUMBER(SEARCH("MAINTAIN",B45))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H52:H64">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0.7"/>
@@ -3233,33 +3426,33 @@
   </cols>
   <sheetData>
     <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="37" t="inlineStr">
+      <c r="B2" s="80" t="inlineStr">
         <is>
           <t>PROFITABILITY  ·  New Compensation Model</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="B3" s="38" t="inlineStr">
+      <c r="B3" s="81" t="inlineStr">
         <is>
           <t>Annual run-rate. Compares the OLD comp model vs the NEW (growth-incentive) model at the intake each one actually drives. Edit yellow (data) and blue (comp terms) cells.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve">  INPUTS</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case value ($)</t>
         </is>
       </c>
-      <c r="E6" s="41">
+      <c r="E6" s="87">
         <f>'Capacity Lite'!E11</f>
         <v/>
       </c>
@@ -3270,13 +3463,13 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case lifespan (months)</t>
         </is>
       </c>
-      <c r="E7" s="43">
-        <f>'Capacity Lite'!E12</f>
+      <c r="E7" s="86">
+        <f>'Capacity Lite'!E13</f>
         <v/>
       </c>
       <c r="G7" s="42" t="inlineStr">
@@ -3286,23 +3479,23 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Max active cases per manager</t>
-        </is>
-      </c>
-      <c r="E8" s="43">
-        <f>'Capacity Lite'!E16</f>
+      <c r="B8" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Effective cases per manager (David's binding)</t>
+        </is>
+      </c>
+      <c r="E8" s="86">
+        <f>'Capacity Lite'!E23</f>
         <v/>
       </c>
       <c r="G8" s="42" t="inlineStr">
         <is>
-          <t>linked (≈143)</t>
+          <t>binding cases/mgr from Capacity Lite (David's ~90)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Collection rate (% of signed value)</t>
         </is>
@@ -3317,7 +3510,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake UNDER OLD comp (cases/week)</t>
         </is>
@@ -3332,7 +3525,7 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="40" t="inlineStr">
+      <c r="B11" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake UNDER NEW comp (cases/week)</t>
         </is>
@@ -3347,7 +3540,7 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — OLD ($/yr)</t>
         </is>
@@ -3362,7 +3555,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="40" t="inlineStr">
+      <c r="B13" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — NEW ($/yr)</t>
         </is>
@@ -3377,7 +3570,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="40" t="inlineStr">
+      <c r="B14" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  James commission — NEW (% of signed value)</t>
         </is>
@@ -3392,7 +3585,7 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Number of sales reps</t>
         </is>
@@ -3403,7 +3596,7 @@
       <c r="G15" s="42" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rep base — OLD ($/yr each)</t>
         </is>
@@ -3414,7 +3607,7 @@
       <c r="G16" s="42" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="40" t="inlineStr">
+      <c r="B17" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rep base — NEW ($/yr each)</t>
         </is>
@@ -3425,7 +3618,7 @@
       <c r="G17" s="42" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="40" t="inlineStr">
+      <c r="B18" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Reps commission — NEW (% pooled)</t>
         </is>
@@ -3440,12 +3633,12 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="40" t="inlineStr">
+      <c r="B19" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case manager loaded comp ($/yr)</t>
         </is>
       </c>
-      <c r="E19" s="50" t="n">
+      <c r="E19" s="84" t="n">
         <v>75000</v>
       </c>
       <c r="G19" s="42" t="inlineStr">
@@ -3455,12 +3648,12 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="40" t="inlineStr">
+      <c r="B20" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead — fixed ($/yr)</t>
         </is>
       </c>
-      <c r="E20" s="50" t="n">
+      <c r="E20" s="84" t="n">
         <v>300000</v>
       </c>
       <c r="G20" s="42" t="inlineStr">
@@ -3470,7 +3663,7 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="40" t="inlineStr">
+      <c r="B21" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead — variable (% of collected rev)</t>
         </is>
@@ -3485,7 +3678,7 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="51" t="inlineStr">
+      <c r="B23" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  ANNUAL RUN-RATE P&amp;L</t>
         </is>
@@ -3514,7 +3707,7 @@
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="B25" s="40" t="inlineStr">
+      <c r="B25" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake (cases/week)</t>
         </is>
@@ -3534,16 +3727,16 @@
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="B26" s="40" t="inlineStr">
+      <c r="B26" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Annual signed case value</t>
         </is>
       </c>
-      <c r="E26" s="56">
+      <c r="E26" s="94">
         <f>(E10*52*E6)</f>
         <v/>
       </c>
-      <c r="G26" s="56">
+      <c r="G26" s="94">
         <f>(E11*52*E6)</f>
         <v/>
       </c>
@@ -3554,16 +3747,16 @@
       </c>
     </row>
     <row r="27" ht="19" customHeight="1">
-      <c r="B27" s="40" t="inlineStr">
+      <c r="B27" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Collected revenue</t>
         </is>
       </c>
-      <c r="E27" s="56">
+      <c r="E27" s="94">
         <f>(E10*52*E6)*E9</f>
         <v/>
       </c>
-      <c r="G27" s="56">
+      <c r="G27" s="94">
         <f>(E11*52*E6)*E9</f>
         <v/>
       </c>
@@ -3574,7 +3767,7 @@
       </c>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="B28" s="40" t="inlineStr">
+      <c r="B28" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case managers required (FTE)</t>
         </is>
@@ -3594,16 +3787,16 @@
       </c>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="B29" s="40" t="inlineStr">
+      <c r="B29" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case manager cost</t>
         </is>
       </c>
-      <c r="E29" s="56">
+      <c r="E29" s="94">
         <f>-((E10*52*(E7/12))/E8*E19)</f>
         <v/>
       </c>
-      <c r="G29" s="56">
+      <c r="G29" s="94">
         <f>-((E11*52*(E7/12))/E8*E19)</f>
         <v/>
       </c>
@@ -3614,16 +3807,16 @@
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="B30" s="40" t="inlineStr">
+      <c r="B30" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  James pay</t>
         </is>
       </c>
-      <c r="E30" s="56">
+      <c r="E30" s="94">
         <f>-E12</f>
         <v/>
       </c>
-      <c r="G30" s="56">
+      <c r="G30" s="94">
         <f>-(E13+E14*(E11*52*E6))</f>
         <v/>
       </c>
@@ -3634,16 +3827,16 @@
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="40" t="inlineStr">
+      <c r="B31" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sales reps pay</t>
         </is>
       </c>
-      <c r="E31" s="56">
+      <c r="E31" s="94">
         <f>-(E15*E16)</f>
         <v/>
       </c>
-      <c r="G31" s="56">
+      <c r="G31" s="94">
         <f>-(E15*E17+E18*(E11*52*E6))</f>
         <v/>
       </c>
@@ -3654,16 +3847,16 @@
       </c>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="B32" s="40" t="inlineStr">
+      <c r="B32" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead</t>
         </is>
       </c>
-      <c r="E32" s="56">
+      <c r="E32" s="94">
         <f>-(E20+E21*((E10*52*E6)*E9))</f>
         <v/>
       </c>
-      <c r="G32" s="56">
+      <c r="G32" s="94">
         <f>-(E20+E21*((E11*52*E6)*E9))</f>
         <v/>
       </c>
@@ -3674,16 +3867,16 @@
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="57" t="inlineStr">
+      <c r="B33" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  NET PROFIT</t>
         </is>
       </c>
-      <c r="E33" s="58">
+      <c r="E33" s="99">
         <f>(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
         <v/>
       </c>
-      <c r="G33" s="58">
+      <c r="G33" s="99">
         <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))</f>
         <v/>
       </c>
@@ -3694,7 +3887,7 @@
       </c>
     </row>
     <row r="34" ht="19" customHeight="1">
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  Net margin</t>
         </is>
@@ -3710,7 +3903,7 @@
       <c r="H34" s="42" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="60" t="inlineStr">
+      <c r="B36" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">  PROFITABILITY IMPACT OF THE NEW COMP MODEL</t>
         </is>
@@ -3722,11 +3915,11 @@
           <t xml:space="preserve">  Δ Collected revenue (new − old)</t>
         </is>
       </c>
-      <c r="E37" s="56">
+      <c r="E37" s="94">
         <f>((E11*52*E6)*E9)-((E10*52*E6)*E9)</f>
         <v/>
       </c>
-      <c r="G37" s="62" t="inlineStr">
+      <c r="G37" s="103" t="inlineStr">
         <is>
           <t>the growth the incentive unlocks</t>
         </is>
@@ -3738,11 +3931,11 @@
           <t xml:space="preserve">  Δ Selling comp cost (new − old)</t>
         </is>
       </c>
-      <c r="E38" s="56">
+      <c r="E38" s="94">
         <f>-(((E13+E14*(E11*52*E6))+(E15*E17+E18*(E11*52*E6)))-(E12+(E15*E16)))</f>
         <v/>
       </c>
-      <c r="G38" s="62" t="inlineStr">
+      <c r="G38" s="103" t="inlineStr">
         <is>
           <t>extra commission the firm pays out</t>
         </is>
@@ -3754,11 +3947,11 @@
           <t xml:space="preserve">  Δ NET PROFIT (new − old)</t>
         </is>
       </c>
-      <c r="E39" s="64">
+      <c r="E39" s="102">
         <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))-(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
         <v/>
       </c>
-      <c r="G39" s="62" t="inlineStr">
+      <c r="G39" s="103" t="inlineStr">
         <is>
           <t>bottom-line effect of switching</t>
         </is>
@@ -3786,7 +3979,7 @@
       <c r="H42" s="36" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="51" t="inlineStr">
+      <c r="B44" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
         </is>
@@ -3922,7 +4115,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="37" t="inlineStr">
+      <c r="B2" s="80" t="inlineStr">
         <is>
           <t>WHY THE NEW MODEL PAYS JAMES MORE</t>
         </is>
@@ -3936,7 +4129,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="57" t="inlineStr">
+      <c r="B5" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — OLD</t>
         </is>
@@ -3945,7 +4138,7 @@
         <f>'Profitability'!E12</f>
         <v/>
       </c>
-      <c r="E5" s="57" t="inlineStr">
+      <c r="E5" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  Target intake (cases/wk)</t>
         </is>
@@ -3956,7 +4149,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — NEW</t>
         </is>
@@ -3967,7 +4160,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="57" t="inlineStr">
+      <c r="B7" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  Commission % (signed value)</t>
         </is>
@@ -3978,7 +4171,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="101" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case value</t>
         </is>
@@ -4019,11 +4212,11 @@
       <c r="B12" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="56">
+      <c r="C12" s="94">
         <f>B12*52*$C$8</f>
         <v/>
       </c>
-      <c r="D12" s="56">
+      <c r="D12" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4031,7 +4224,7 @@
         <f>$C$6+$C$7*C12</f>
         <v/>
       </c>
-      <c r="F12" s="56">
+      <c r="F12" s="94">
         <f>E12-D12</f>
         <v/>
       </c>
@@ -4040,11 +4233,11 @@
       <c r="B13" s="55" t="n">
         <v>2.5</v>
       </c>
-      <c r="C13" s="56">
+      <c r="C13" s="94">
         <f>B13*52*$C$8</f>
         <v/>
       </c>
-      <c r="D13" s="56">
+      <c r="D13" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4052,7 +4245,7 @@
         <f>$C$6+$C$7*C13</f>
         <v/>
       </c>
-      <c r="F13" s="56">
+      <c r="F13" s="94">
         <f>E13-D13</f>
         <v/>
       </c>
@@ -4061,11 +4254,11 @@
       <c r="B14" s="55" t="n">
         <v>5</v>
       </c>
-      <c r="C14" s="56">
+      <c r="C14" s="94">
         <f>B14*52*$C$8</f>
         <v/>
       </c>
-      <c r="D14" s="56">
+      <c r="D14" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4073,7 +4266,7 @@
         <f>$C$6+$C$7*C14</f>
         <v/>
       </c>
-      <c r="F14" s="56">
+      <c r="F14" s="94">
         <f>E14-D14</f>
         <v/>
       </c>
@@ -4082,11 +4275,11 @@
       <c r="B15" s="55" t="n">
         <v>7.5</v>
       </c>
-      <c r="C15" s="56">
+      <c r="C15" s="94">
         <f>B15*52*$C$8</f>
         <v/>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4094,7 +4287,7 @@
         <f>$C$6+$C$7*C15</f>
         <v/>
       </c>
-      <c r="F15" s="56">
+      <c r="F15" s="94">
         <f>E15-D15</f>
         <v/>
       </c>
@@ -4103,11 +4296,11 @@
       <c r="B16" s="55" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="94">
         <f>B16*52*$C$8</f>
         <v/>
       </c>
-      <c r="D16" s="56">
+      <c r="D16" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4115,7 +4308,7 @@
         <f>$C$6+$C$7*C16</f>
         <v/>
       </c>
-      <c r="F16" s="56">
+      <c r="F16" s="94">
         <f>E16-D16</f>
         <v/>
       </c>
@@ -4124,11 +4317,11 @@
       <c r="B17" s="55" t="n">
         <v>12.5</v>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="94">
         <f>B17*52*$C$8</f>
         <v/>
       </c>
-      <c r="D17" s="56">
+      <c r="D17" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4136,7 +4329,7 @@
         <f>$C$6+$C$7*C17</f>
         <v/>
       </c>
-      <c r="F17" s="56">
+      <c r="F17" s="94">
         <f>E17-D17</f>
         <v/>
       </c>
@@ -4145,11 +4338,11 @@
       <c r="B18" s="55" t="n">
         <v>15</v>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="94">
         <f>B18*52*$C$8</f>
         <v/>
       </c>
-      <c r="D18" s="56">
+      <c r="D18" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4157,7 +4350,7 @@
         <f>$C$6+$C$7*C18</f>
         <v/>
       </c>
-      <c r="F18" s="56">
+      <c r="F18" s="94">
         <f>E18-D18</f>
         <v/>
       </c>
@@ -4166,11 +4359,11 @@
       <c r="B19" s="55" t="n">
         <v>17.5</v>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="94">
         <f>B19*52*$C$8</f>
         <v/>
       </c>
-      <c r="D19" s="56">
+      <c r="D19" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4178,7 +4371,7 @@
         <f>$C$6+$C$7*C19</f>
         <v/>
       </c>
-      <c r="F19" s="56">
+      <c r="F19" s="94">
         <f>E19-D19</f>
         <v/>
       </c>
@@ -4187,11 +4380,11 @@
       <c r="B20" s="55" t="n">
         <v>20</v>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="94">
         <f>B20*52*$C$8</f>
         <v/>
       </c>
-      <c r="D20" s="56">
+      <c r="D20" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4199,7 +4392,7 @@
         <f>$C$6+$C$7*C20</f>
         <v/>
       </c>
-      <c r="F20" s="56">
+      <c r="F20" s="94">
         <f>E20-D20</f>
         <v/>
       </c>
@@ -4208,11 +4401,11 @@
       <c r="B21" s="55" t="n">
         <v>22.5</v>
       </c>
-      <c r="C21" s="56">
+      <c r="C21" s="94">
         <f>B21*52*$C$8</f>
         <v/>
       </c>
-      <c r="D21" s="56">
+      <c r="D21" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4220,7 +4413,7 @@
         <f>$C$6+$C$7*C21</f>
         <v/>
       </c>
-      <c r="F21" s="56">
+      <c r="F21" s="94">
         <f>E21-D21</f>
         <v/>
       </c>
@@ -4250,11 +4443,11 @@
       <c r="B23" s="55" t="n">
         <v>27.5</v>
       </c>
-      <c r="C23" s="56">
+      <c r="C23" s="94">
         <f>B23*52*$C$8</f>
         <v/>
       </c>
-      <c r="D23" s="56">
+      <c r="D23" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4262,7 +4455,7 @@
         <f>$C$6+$C$7*C23</f>
         <v/>
       </c>
-      <c r="F23" s="56">
+      <c r="F23" s="94">
         <f>E23-D23</f>
         <v/>
       </c>
@@ -4271,11 +4464,11 @@
       <c r="B24" s="55" t="n">
         <v>30</v>
       </c>
-      <c r="C24" s="56">
+      <c r="C24" s="94">
         <f>B24*52*$C$8</f>
         <v/>
       </c>
-      <c r="D24" s="56">
+      <c r="D24" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4283,7 +4476,7 @@
         <f>$C$6+$C$7*C24</f>
         <v/>
       </c>
-      <c r="F24" s="56">
+      <c r="F24" s="94">
         <f>E24-D24</f>
         <v/>
       </c>
@@ -4292,11 +4485,11 @@
       <c r="B25" s="55" t="n">
         <v>32.5</v>
       </c>
-      <c r="C25" s="56">
+      <c r="C25" s="94">
         <f>B25*52*$C$8</f>
         <v/>
       </c>
-      <c r="D25" s="56">
+      <c r="D25" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4304,7 +4497,7 @@
         <f>$C$6+$C$7*C25</f>
         <v/>
       </c>
-      <c r="F25" s="56">
+      <c r="F25" s="94">
         <f>E25-D25</f>
         <v/>
       </c>
@@ -4313,11 +4506,11 @@
       <c r="B26" s="55" t="n">
         <v>35</v>
       </c>
-      <c r="C26" s="56">
+      <c r="C26" s="94">
         <f>B26*52*$C$8</f>
         <v/>
       </c>
-      <c r="D26" s="56">
+      <c r="D26" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4325,7 +4518,7 @@
         <f>$C$6+$C$7*C26</f>
         <v/>
       </c>
-      <c r="F26" s="56">
+      <c r="F26" s="94">
         <f>E26-D26</f>
         <v/>
       </c>
@@ -4334,11 +4527,11 @@
       <c r="B27" s="55" t="n">
         <v>37.5</v>
       </c>
-      <c r="C27" s="56">
+      <c r="C27" s="94">
         <f>B27*52*$C$8</f>
         <v/>
       </c>
-      <c r="D27" s="56">
+      <c r="D27" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4346,7 +4539,7 @@
         <f>$C$6+$C$7*C27</f>
         <v/>
       </c>
-      <c r="F27" s="56">
+      <c r="F27" s="94">
         <f>E27-D27</f>
         <v/>
       </c>
@@ -4355,11 +4548,11 @@
       <c r="B28" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="C28" s="56">
+      <c r="C28" s="94">
         <f>B28*52*$C$8</f>
         <v/>
       </c>
-      <c r="D28" s="56">
+      <c r="D28" s="94">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4367,7 +4560,7 @@
         <f>$C$6+$C$7*C28</f>
         <v/>
       </c>
-      <c r="F28" s="56">
+      <c r="F28" s="94">
         <f>E28-D28</f>
         <v/>
       </c>
@@ -5441,8 +5634,28 @@
         <f>IF(MIN(J23:J40)&lt;0,"CASH GOES NEGATIVE DURING RAMP — secure a buffer / line of credit before scaling intake","CASH STAYS POSITIVE — but early months bank well below run-rate; keep the buffer intact")</f>
         <v/>
       </c>
-    </row>
-    <row r="46"/>
+      <c r="C45" s="30" t="n"/>
+      <c r="D45" s="30" t="n"/>
+      <c r="E45" s="30" t="n"/>
+      <c r="F45" s="30" t="n"/>
+      <c r="G45" s="30" t="n"/>
+      <c r="H45" s="30" t="n"/>
+      <c r="I45" s="30" t="n"/>
+      <c r="J45" s="30" t="n"/>
+      <c r="K45" s="31" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="34" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35" t="n"/>
+      <c r="F46" s="35" t="n"/>
+      <c r="G46" s="35" t="n"/>
+      <c r="H46" s="35" t="n"/>
+      <c r="I46" s="35" t="n"/>
+      <c r="J46" s="35" t="n"/>
+      <c r="K46" s="36" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="23">
     <mergeCell ref="B9:E9"/>
@@ -6004,8 +6217,8 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D13:F13"/>
     <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D13:F13"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B3:F3"/>

</xml_diff>

<commit_message>
Add Org & Hiring Triggers tab from org chart
Builds hiring-trigger logic off the David J Griggs CPA org chart:
four roles, four drivers. Case Managers scale with caseload; Admins
scale with CM count AND lift CM capacity 90->130 (humans-vs-admins
lever); Account Executives scale with monthly intake; Case Directors
scale with management span. Includes current-org table, editable
staffing ratios, live hire-trigger status flags, plain-English next-hire
thresholds, an admin trade-off block, and a 12-month staffing plan +
chart driven by the Capacity Lite projection.
</commit_message>
<xml_diff>
--- a/Capacity-Lite.xlsx
+++ b/Capacity-Lite.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Capacity Lite" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Profitability" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="James — New Comp" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Timing" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comp Optimizer" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Org &amp; Hiring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Profitability" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="James — New Comp" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cash Timing" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Comp Optimizer" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="39">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -219,8 +220,33 @@
       <color rgb="00B3402E"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00455064"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007A8499"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B3402E"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00B3402E"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00101A30"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -265,6 +291,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBECCB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4D8D1"/>
       </patternFill>
     </fill>
   </fills>
@@ -387,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -842,11 +873,92 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="36" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="17">
     <dxf>
       <font>
         <b val="1"/>
@@ -980,6 +1092,39 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00D9ECE2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B3402E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4D8D1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B9831A"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBECCB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C7415"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBECCB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1195,6 +1340,217 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Headcount needed as the book grows</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Org &amp; Hiring'!D54</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="34000">
+              <a:solidFill>
+                <a:srgbClr val="C8961E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Org &amp; Hiring'!$B$55:$B$67</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Org &amp; Hiring'!$D$55:$D$67</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Org &amp; Hiring'!E54</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="26000">
+              <a:solidFill>
+                <a:srgbClr val="1B2A4A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Org &amp; Hiring'!$B$55:$B$67</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Org &amp; Hiring'!$E$55:$E$67</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Org &amp; Hiring'!F54</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="26000">
+              <a:solidFill>
+                <a:srgbClr val="2F7D5B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Org &amp; Hiring'!$B$55:$B$67</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Org &amp; Hiring'!$F$55:$F$67</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Org &amp; Hiring'!G54</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="26000">
+              <a:solidFill>
+                <a:srgbClr val="B3402E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Org &amp; Hiring'!$B$55:$B$67</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Org &amp; Hiring'!$G$55:$G$67</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>People</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>James's annual pay: OLD (flat salary) vs NEW (base + growth commission)</a:t>
             </a:r>
           </a:p>
@@ -1342,7 +1698,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1449,7 +1805,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1611,7 +1967,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1799,6 +2155,33 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>4</row>
@@ -1822,7 +2205,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1871,7 +2254,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -2558,9 +2941,30 @@
         <f>IF(G18&lt;E18,"⚠ CAN'T HIT $1M/MGR AT BASE PRICE — At David's "&amp;TEXT(G18,"0")&amp;" cases/mgr each manager tops out at "&amp;TEXT(G19,"$#,##0")&amp;"/yr. "&amp;TEXT(E20,"0.0")&amp;" FTE = "&amp;TEXT(G22,"$#,##0")&amp;" capacity vs the "&amp;TEXT(E22,"$#,##0")&amp;" target ("&amp;TEXT(E24,"$#,##0")&amp;" short). Fix: raise price to "&amp;TEXT(E25,"$#,##0")&amp;"/case, or add managers, or lower the target.","✓ David's operational capacity supports the revenue target at the current base price.")</f>
         <v/>
       </c>
-    </row>
-    <row r="32" ht="22" customHeight="1"/>
-    <row r="33" ht="22" customHeight="1"/>
+      <c r="C31" s="30" t="n"/>
+      <c r="D31" s="30" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="31" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="32" t="n"/>
+      <c r="J32" s="33" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="34" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="35" t="n"/>
+      <c r="H33" s="35" t="n"/>
+      <c r="I33" s="35" t="n"/>
+      <c r="J33" s="36" t="n"/>
+    </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="119" t="inlineStr">
         <is>
@@ -2701,9 +3105,30 @@
         <f>IF(E37&gt;=E14,"ADD CAPACITY",IF(E37&lt;=E14-0.2,"SELL MORE","MAINTAIN"))</f>
         <v/>
       </c>
-    </row>
-    <row r="46"/>
-    <row r="47"/>
+      <c r="C45" s="30" t="n"/>
+      <c r="D45" s="30" t="n"/>
+      <c r="E45" s="30" t="n"/>
+      <c r="F45" s="30" t="n"/>
+      <c r="G45" s="30" t="n"/>
+      <c r="H45" s="30" t="n"/>
+      <c r="I45" s="30" t="n"/>
+      <c r="J45" s="31" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="32" t="n"/>
+      <c r="J46" s="33" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="34" t="n"/>
+      <c r="C47" s="35" t="n"/>
+      <c r="D47" s="35" t="n"/>
+      <c r="E47" s="35" t="n"/>
+      <c r="F47" s="35" t="n"/>
+      <c r="G47" s="35" t="n"/>
+      <c r="H47" s="35" t="n"/>
+      <c r="I47" s="35" t="n"/>
+      <c r="J47" s="36" t="n"/>
+    </row>
     <row r="48">
       <c r="B48" s="149" t="inlineStr">
         <is>
@@ -3328,8 +3753,8 @@
   <mergeCells count="42">
     <mergeCell ref="B67:J67"/>
     <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G25:J25"/>
     <mergeCell ref="H17:J17"/>
-    <mergeCell ref="G25:J25"/>
     <mergeCell ref="G41:J41"/>
     <mergeCell ref="B69:J69"/>
     <mergeCell ref="G40:J40"/>
@@ -3341,8 +3766,8 @@
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="B30:J30"/>
     <mergeCell ref="G36:J36"/>
+    <mergeCell ref="B68:J68"/>
     <mergeCell ref="G42:J42"/>
-    <mergeCell ref="B68:J68"/>
     <mergeCell ref="B5:J5"/>
     <mergeCell ref="H18:J18"/>
     <mergeCell ref="G23:J23"/>
@@ -3408,6 +3833,1277 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001B2A4A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="158" t="inlineStr">
+        <is>
+          <t>ORG &amp; HIRING TRIGGERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="66" t="inlineStr">
+        <is>
+          <t>When to add each kind of human. Four roles, four different triggers — all driven by the Capacity Lite numbers. Edit the yellow rules; the status flags and 12-month plan recalc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CURRENT ORG  (from David J Griggs CPA org chart, July 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="160" t="inlineStr">
+        <is>
+          <t>Function / Role</t>
+        </is>
+      </c>
+      <c r="C6" s="79" t="n"/>
+      <c r="D6" s="160" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E6" s="79" t="n"/>
+      <c r="F6" s="160" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G6" s="79" t="n"/>
+      <c r="H6" s="161" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CEO</t>
+        </is>
+      </c>
+      <c r="D7" s="163" t="inlineStr">
+        <is>
+          <t>David Griggs</t>
+        </is>
+      </c>
+      <c r="F7" s="164" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H7" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sales management</t>
+        </is>
+      </c>
+      <c r="D8" s="163" t="inlineStr">
+        <is>
+          <t>Josh Alltop</t>
+        </is>
+      </c>
+      <c r="F8" s="164" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="H8" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Account Executive</t>
+        </is>
+      </c>
+      <c r="D9" s="163" t="inlineStr">
+        <is>
+          <t>(new role — hiring)</t>
+        </is>
+      </c>
+      <c r="F9" s="164" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H9" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case Director</t>
+        </is>
+      </c>
+      <c r="D10" s="163" t="inlineStr">
+        <is>
+          <t>James</t>
+        </is>
+      </c>
+      <c r="F10" s="164" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H10" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case Managers</t>
+        </is>
+      </c>
+      <c r="D11" s="163" t="inlineStr">
+        <is>
+          <t>4 × 80–100 accounts</t>
+        </is>
+      </c>
+      <c r="F11" s="164" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H11" s="165" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Admin / case support</t>
+        </is>
+      </c>
+      <c r="D12" s="163" t="inlineStr">
+        <is>
+          <t>— none today —</t>
+        </is>
+      </c>
+      <c r="F12" s="164" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="H12" s="167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Operations (advisory)</t>
+        </is>
+      </c>
+      <c r="D13" s="163" t="inlineStr">
+        <is>
+          <t>Denise O'Donnell</t>
+        </is>
+      </c>
+      <c r="F13" s="164" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="H13" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Strategy &amp; HR (advisory)</t>
+        </is>
+      </c>
+      <c r="D14" s="163" t="inlineStr">
+        <is>
+          <t>Vanessa Esquivel</t>
+        </is>
+      </c>
+      <c r="F14" s="164" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="H14" s="165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ► No dedicated admin today — this is why case managers cap at ~90 accounts, not the ~130 they carried WITH admin support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STAFFING RULES &amp; CURRENT COUNTS  (yellow = editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cases per manager — no admin</t>
+        </is>
+      </c>
+      <c r="E18" s="170">
+        <f>'Capacity Lite'!E12</f>
+        <v/>
+      </c>
+      <c r="F18" s="171" t="inlineStr">
+        <is>
+          <t>David's operational estimate (linked)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cases per manager — with full admin</t>
+        </is>
+      </c>
+      <c r="E19" s="172" t="n">
+        <v>130</v>
+      </c>
+      <c r="F19" s="171" t="inlineStr">
+        <is>
+          <t>the 130 historical, with support</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case managers per admin</t>
+        </is>
+      </c>
+      <c r="E20" s="172" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="171" t="inlineStr">
+        <is>
+          <t>how many CMs one admin supports</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New cases / month one AE can close</t>
+        </is>
+      </c>
+      <c r="E21" s="172" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" s="171" t="inlineStr">
+        <is>
+          <t>sales throughput per Account Executive</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case managers per Case Director (span)</t>
+        </is>
+      </c>
+      <c r="E22" s="172" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" s="171" t="inlineStr">
+        <is>
+          <t>management span of control</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current case managers</t>
+        </is>
+      </c>
+      <c r="E23" s="172" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="171" t="inlineStr">
+        <is>
+          <t>from org chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current admins</t>
+        </is>
+      </c>
+      <c r="E24" s="172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="171" t="inlineStr">
+        <is>
+          <t>from org chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current Account Executives</t>
+        </is>
+      </c>
+      <c r="E25" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="171" t="inlineStr">
+        <is>
+          <t>incl. the new hire</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current Case Directors</t>
+        </is>
+      </c>
+      <c r="E26" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="171" t="inlineStr">
+        <is>
+          <t>James</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hire trigger (utilization)</t>
+        </is>
+      </c>
+      <c r="E27" s="173">
+        <f>'Capacity Lite'!E14</f>
+        <v/>
+      </c>
+      <c r="F27" s="171" t="inlineStr">
+        <is>
+          <t>hire before crossing this (linked)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DRIVERS &amp; EFFECTIVE CAPACITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current open cases</t>
+        </is>
+      </c>
+      <c r="E30" s="174">
+        <f>'Capacity Lite'!E8</f>
+        <v/>
+      </c>
+      <c r="F30" s="171" t="inlineStr">
+        <is>
+          <t>linked from Capacity Lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New cases / month</t>
+        </is>
+      </c>
+      <c r="E31" s="175">
+        <f>'Capacity Lite'!E40</f>
+        <v/>
+      </c>
+      <c r="F31" s="171" t="inlineStr">
+        <is>
+          <t>linked from Capacity Lite</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Effective cases / manager (with current admin)</t>
+        </is>
+      </c>
+      <c r="E32" s="176">
+        <f>E18+(E19-E18)*MIN(1,E24/ROUNDUP(E23/E20,0))</f>
+        <v/>
+      </c>
+      <c r="F32" s="177" t="inlineStr">
+        <is>
+          <t>admin coverage lifts CM capacity 90→130</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HIRE TRIGGERS  —  where you stand right now</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>Capacity each</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="inlineStr">
+        <is>
+          <t>Need (to comfort)</t>
+        </is>
+      </c>
+      <c r="F35" s="20" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="G35" s="20" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="H35" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case Managers</t>
+        </is>
+      </c>
+      <c r="C36" s="178">
+        <f>"open cases"</f>
+        <v/>
+      </c>
+      <c r="D36" s="179">
+        <f>E32</f>
+        <v/>
+      </c>
+      <c r="E36" s="165">
+        <f>ROUNDUP('Capacity Lite'!E8/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="F36" s="180">
+        <f>E23</f>
+        <v/>
+      </c>
+      <c r="G36" s="165">
+        <f>E36-F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="181">
+        <f>IF('Capacity Lite'!E8/(E23*E32)&gt;1,"HIRE NOW",IF('Capacity Lite'!E8/(E23*E32)&gt;E27,"HIRE SOON","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Admins</t>
+        </is>
+      </c>
+      <c r="C37" s="178">
+        <f>"case mgrs"</f>
+        <v/>
+      </c>
+      <c r="D37" s="179">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="E37" s="165">
+        <f>ROUNDUP(E23/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F37" s="180">
+        <f>E24</f>
+        <v/>
+      </c>
+      <c r="G37" s="165">
+        <f>E37-F37</f>
+        <v/>
+      </c>
+      <c r="H37" s="181">
+        <f>IF(E24&lt;ROUNDUP(E23/E20,0),"HIRE NOW","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Account Executives</t>
+        </is>
+      </c>
+      <c r="C38" s="178">
+        <f>"new/mo"</f>
+        <v/>
+      </c>
+      <c r="D38" s="179">
+        <f>E21</f>
+        <v/>
+      </c>
+      <c r="E38" s="165">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="180">
+        <f>E25</f>
+        <v/>
+      </c>
+      <c r="G38" s="165">
+        <f>E38-F38</f>
+        <v/>
+      </c>
+      <c r="H38" s="181">
+        <f>IF(E25&lt;ROUNDUP('Capacity Lite'!E40/E21,0),"HIRE NOW","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case Directors</t>
+        </is>
+      </c>
+      <c r="C39" s="178">
+        <f>"case mgrs"</f>
+        <v/>
+      </c>
+      <c r="D39" s="179">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="E39" s="165">
+        <f>ROUNDUP(E23/E22,0)</f>
+        <v/>
+      </c>
+      <c r="F39" s="180">
+        <f>E26</f>
+        <v/>
+      </c>
+      <c r="G39" s="165">
+        <f>E39-F39</f>
+        <v/>
+      </c>
+      <c r="H39" s="181">
+        <f>IF(E26&lt;ROUNDUP(E23/E22,0),"HIRE","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="B41" s="159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NEXT-HIRE THRESHOLDS  (plain English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="182">
+        <f>CONCATENATE("Add Case Manager #",TEXT(E23+1,"0")," when open cases exceed ",TEXT(E23*E32*E27,"0")," (comfort) — hard ceiling ",TEXT(E23*E32,"0"),".")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="182">
+        <f>CONCATENATE("Add your 1st/next Admin when case managers reach ",TEXT((E24+1)*E20,"0"),". Each admin lifts CM capacity toward ",TEXT(E19,"0")," accounts.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="182">
+        <f>CONCATENATE("Add Account Executive #",TEXT(E25+1,"0")," when new cases/month exceed ",TEXT(E25*E21,"0"),". You are at ",TEXT('Capacity Lite'!E40,"0"),"/mo now.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="182">
+        <f>CONCATENATE("Add a 2nd Case Director when case managers exceed ",TEXT(E22*E26,"0"),".")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="B47" s="169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HUMANS vs ADMINS — the capacity lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case managers to carry today's book — NO admin (90)</t>
+        </is>
+      </c>
+      <c r="E48" s="183">
+        <f>ROUNDUP('Capacity Lite'!E8/E18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Case managers — WITH full admin (130)</t>
+        </is>
+      </c>
+      <c r="E49" s="183">
+        <f>ROUNDUP('Capacity Lite'!E8/E19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Admins needed for that full-support level</t>
+        </is>
+      </c>
+      <c r="E50" s="183">
+        <f>ROUNDUP(E49/E20,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="184">
+        <f>CONCATENATE("► Adding ",TEXT(E50,"0")," admin(s) lets ",TEXT(E48-E49,"0")," fewer case manager(s) carry the same book. Admins are the cheaper capacity lever until you outgrow them.")</f>
+        <v/>
+      </c>
+      <c r="C51" s="78" t="n"/>
+      <c r="D51" s="78" t="n"/>
+      <c r="E51" s="78" t="n"/>
+      <c r="F51" s="78" t="n"/>
+      <c r="G51" s="78" t="n"/>
+      <c r="H51" s="78" t="n"/>
+      <c r="I51" s="79" t="n"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="B53" s="159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  12-MONTH STAFFING PLAN  (headcount needed as the book grows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>Open cases</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>Case Mgrs</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>Admins</t>
+        </is>
+      </c>
+      <c r="F54" s="20" t="inlineStr">
+        <is>
+          <t>Account Execs</t>
+        </is>
+      </c>
+      <c r="G54" s="20" t="inlineStr">
+        <is>
+          <t>Case Directors</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="B55" s="181" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C55" s="180">
+        <f>'Capacity Lite'!F52</f>
+        <v/>
+      </c>
+      <c r="D55" s="165">
+        <f>ROUNDUP('Capacity Lite'!F52/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E55" s="180">
+        <f>ROUNDUP(D55/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F55" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="180">
+        <f>ROUNDUP(D55/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="B56" s="178" t="inlineStr">
+        <is>
+          <t>Mo 1</t>
+        </is>
+      </c>
+      <c r="C56" s="180">
+        <f>'Capacity Lite'!F53</f>
+        <v/>
+      </c>
+      <c r="D56" s="165">
+        <f>ROUNDUP('Capacity Lite'!F53/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E56" s="180">
+        <f>ROUNDUP(D56/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F56" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="180">
+        <f>ROUNDUP(D56/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="B57" s="178" t="inlineStr">
+        <is>
+          <t>Mo 2</t>
+        </is>
+      </c>
+      <c r="C57" s="180">
+        <f>'Capacity Lite'!F54</f>
+        <v/>
+      </c>
+      <c r="D57" s="165">
+        <f>ROUNDUP('Capacity Lite'!F54/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E57" s="180">
+        <f>ROUNDUP(D57/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F57" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="180">
+        <f>ROUNDUP(D57/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="B58" s="178" t="inlineStr">
+        <is>
+          <t>Mo 3</t>
+        </is>
+      </c>
+      <c r="C58" s="180">
+        <f>'Capacity Lite'!F55</f>
+        <v/>
+      </c>
+      <c r="D58" s="165">
+        <f>ROUNDUP('Capacity Lite'!F55/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E58" s="180">
+        <f>ROUNDUP(D58/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F58" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="180">
+        <f>ROUNDUP(D58/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="B59" s="178" t="inlineStr">
+        <is>
+          <t>Mo 4</t>
+        </is>
+      </c>
+      <c r="C59" s="180">
+        <f>'Capacity Lite'!F56</f>
+        <v/>
+      </c>
+      <c r="D59" s="165">
+        <f>ROUNDUP('Capacity Lite'!F56/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E59" s="180">
+        <f>ROUNDUP(D59/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F59" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="180">
+        <f>ROUNDUP(D59/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="B60" s="178" t="inlineStr">
+        <is>
+          <t>Mo 5</t>
+        </is>
+      </c>
+      <c r="C60" s="180">
+        <f>'Capacity Lite'!F57</f>
+        <v/>
+      </c>
+      <c r="D60" s="165">
+        <f>ROUNDUP('Capacity Lite'!F57/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E60" s="180">
+        <f>ROUNDUP(D60/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F60" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="180">
+        <f>ROUNDUP(D60/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="B61" s="178" t="inlineStr">
+        <is>
+          <t>Mo 6</t>
+        </is>
+      </c>
+      <c r="C61" s="180">
+        <f>'Capacity Lite'!F58</f>
+        <v/>
+      </c>
+      <c r="D61" s="165">
+        <f>ROUNDUP('Capacity Lite'!F58/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E61" s="180">
+        <f>ROUNDUP(D61/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F61" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="180">
+        <f>ROUNDUP(D61/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="B62" s="178" t="inlineStr">
+        <is>
+          <t>Mo 7</t>
+        </is>
+      </c>
+      <c r="C62" s="180">
+        <f>'Capacity Lite'!F59</f>
+        <v/>
+      </c>
+      <c r="D62" s="165">
+        <f>ROUNDUP('Capacity Lite'!F59/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E62" s="180">
+        <f>ROUNDUP(D62/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F62" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="180">
+        <f>ROUNDUP(D62/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="B63" s="178" t="inlineStr">
+        <is>
+          <t>Mo 8</t>
+        </is>
+      </c>
+      <c r="C63" s="180">
+        <f>'Capacity Lite'!F60</f>
+        <v/>
+      </c>
+      <c r="D63" s="165">
+        <f>ROUNDUP('Capacity Lite'!F60/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E63" s="180">
+        <f>ROUNDUP(D63/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F63" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="180">
+        <f>ROUNDUP(D63/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="B64" s="178" t="inlineStr">
+        <is>
+          <t>Mo 9</t>
+        </is>
+      </c>
+      <c r="C64" s="180">
+        <f>'Capacity Lite'!F61</f>
+        <v/>
+      </c>
+      <c r="D64" s="165">
+        <f>ROUNDUP('Capacity Lite'!F61/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E64" s="180">
+        <f>ROUNDUP(D64/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F64" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="180">
+        <f>ROUNDUP(D64/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="B65" s="178" t="inlineStr">
+        <is>
+          <t>Mo 10</t>
+        </is>
+      </c>
+      <c r="C65" s="180">
+        <f>'Capacity Lite'!F62</f>
+        <v/>
+      </c>
+      <c r="D65" s="165">
+        <f>ROUNDUP('Capacity Lite'!F62/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E65" s="180">
+        <f>ROUNDUP(D65/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F65" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="180">
+        <f>ROUNDUP(D65/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="15" customHeight="1">
+      <c r="B66" s="178" t="inlineStr">
+        <is>
+          <t>Mo 11</t>
+        </is>
+      </c>
+      <c r="C66" s="180">
+        <f>'Capacity Lite'!F63</f>
+        <v/>
+      </c>
+      <c r="D66" s="165">
+        <f>ROUNDUP('Capacity Lite'!F63/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E66" s="180">
+        <f>ROUNDUP(D66/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F66" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="180">
+        <f>ROUNDUP(D66/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="B67" s="178" t="inlineStr">
+        <is>
+          <t>Mo 12</t>
+        </is>
+      </c>
+      <c r="C67" s="180">
+        <f>'Capacity Lite'!F64</f>
+        <v/>
+      </c>
+      <c r="D67" s="165">
+        <f>ROUNDUP('Capacity Lite'!F64/(E32*E27),0)</f>
+        <v/>
+      </c>
+      <c r="E67" s="180">
+        <f>ROUNDUP(D67/E20,0)</f>
+        <v/>
+      </c>
+      <c r="F67" s="180">
+        <f>ROUNDUP('Capacity Lite'!E40/E21,0)</f>
+        <v/>
+      </c>
+      <c r="G67" s="180">
+        <f>ROUNDUP(D67/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="B69" s="169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="B70" s="29" t="inlineStr">
+        <is>
+          <t>•  Four triggers, four drivers: Case Managers scale with caseload; Admins scale with case-manager count (and raise CM capacity 90→130); Account Executives scale with monthly intake; Case Directors scale with management span.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="B71" s="29" t="inlineStr">
+        <is>
+          <t>•  Admins are a capacity multiplier, not just overhead — before hiring the next case manager, check whether an admin (cheaper) buys enough headroom. That is the humans-vs-admins lever.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="B72" s="29" t="inlineStr">
+        <is>
+          <t>•  The 12-month plan reads today's open-case projection off Capacity Lite; where a case-manager count steps up (highlighted) is when to have the hire ramped and ready — start recruiting 1–2 months earlier given onboarding lead time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>•  Ratios (cases/mgr, CMs per admin, AE throughput, span) are starting placeholders — set them to David's real numbers. Org counts are from the July 2026 chart; both draft versions have the same headcount (they differ only in the AE's reporting line).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="B74" s="29" t="inlineStr">
+        <is>
+          <t>•  Josh, Denise and Vanessa are contractors today — the model counts them as 1 each; convert to FTE triggers separately if/when advisory load justifies it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="61">
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="B47:I47"/>
+    <mergeCell ref="B72:I72"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B71:I71"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B70:I70"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B73:I73"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B69:I69"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F22:I22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="expression" priority="1" dxfId="14">
+      <formula>ISNUMBER(SEARCH("NOW",H36))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="15">
+      <formula>ISNUMBER(SEARCH("SOON",H36))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="10">
+      <formula>EXACT(H36,"OK")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36">
+    <cfRule type="expression" priority="4" dxfId="7">
+      <formula>G36&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="expression" priority="5" dxfId="14">
+      <formula>ISNUMBER(SEARCH("NOW",H37))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="15">
+      <formula>ISNUMBER(SEARCH("SOON",H37))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="10">
+      <formula>EXACT(H37,"OK")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
+    <cfRule type="expression" priority="8" dxfId="7">
+      <formula>G37&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="expression" priority="9" dxfId="14">
+      <formula>ISNUMBER(SEARCH("NOW",H38))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="15">
+      <formula>ISNUMBER(SEARCH("SOON",H38))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="10">
+      <formula>EXACT(H38,"OK")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G38">
+    <cfRule type="expression" priority="12" dxfId="7">
+      <formula>G38&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H39">
+    <cfRule type="expression" priority="13" dxfId="14">
+      <formula>ISNUMBER(SEARCH("NOW",H39))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="15">
+      <formula>ISNUMBER(SEARCH("SOON",H39))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="10">
+      <formula>EXACT(H39,"OK")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G39">
+    <cfRule type="expression" priority="16" dxfId="7">
+      <formula>G39&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D56:D67">
+    <cfRule type="expression" priority="17" dxfId="16">
+      <formula>D56&gt;D55</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="002F7D5B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3440,14 +5136,14 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="82" t="inlineStr">
+      <c r="B5" s="119" t="inlineStr">
         <is>
           <t xml:space="preserve">  INPUTS</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="106" t="inlineStr">
+      <c r="B6" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case value ($)</t>
         </is>
@@ -3456,14 +5152,14 @@
         <f>'Capacity Lite'!E11</f>
         <v/>
       </c>
-      <c r="G6" s="42" t="inlineStr">
+      <c r="G6" s="135" t="inlineStr">
         <is>
           <t>linked from Capacity Lite</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="B7" s="106" t="inlineStr">
+      <c r="B7" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Average case lifespan (months)</t>
         </is>
@@ -3472,14 +5168,14 @@
         <f>'Capacity Lite'!E13</f>
         <v/>
       </c>
-      <c r="G7" s="42" t="inlineStr">
+      <c r="G7" s="135" t="inlineStr">
         <is>
           <t>linked from Capacity Lite</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="106" t="inlineStr">
+      <c r="B8" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Effective cases per manager (David's binding)</t>
         </is>
@@ -3488,14 +5184,14 @@
         <f>'Capacity Lite'!E23</f>
         <v/>
       </c>
-      <c r="G8" s="42" t="inlineStr">
+      <c r="G8" s="135" t="inlineStr">
         <is>
           <t>binding cases/mgr from Capacity Lite (David's ~90)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="106" t="inlineStr">
+      <c r="B9" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Collection rate (% of signed value)</t>
         </is>
@@ -3503,14 +5199,14 @@
       <c r="E9" s="44" t="n">
         <v>0.85</v>
       </c>
-      <c r="G9" s="42" t="inlineStr">
+      <c r="G9" s="135" t="inlineStr">
         <is>
           <t>share of signed fees actually collected</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="106" t="inlineStr">
+      <c r="B10" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake UNDER OLD comp (cases/week)</t>
         </is>
@@ -3518,14 +5214,14 @@
       <c r="E10" s="45" t="n">
         <v>12</v>
       </c>
-      <c r="G10" s="42" t="inlineStr">
+      <c r="G10" s="135" t="inlineStr">
         <is>
           <t>what James/reps produce on salary</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="106" t="inlineStr">
+      <c r="B11" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake UNDER NEW comp (cases/week)</t>
         </is>
@@ -3533,14 +5229,14 @@
       <c r="E11" s="45" t="n">
         <v>25</v>
       </c>
-      <c r="G11" s="42" t="inlineStr">
+      <c r="G11" s="135" t="inlineStr">
         <is>
           <t>the incentivized target: 3 reps + James</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="106" t="inlineStr">
+      <c r="B12" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — OLD ($/yr)</t>
         </is>
@@ -3548,14 +5244,14 @@
       <c r="E12" s="46" t="n">
         <v>90000</v>
       </c>
-      <c r="G12" s="42" t="inlineStr">
+      <c r="G12" s="135" t="inlineStr">
         <is>
           <t>salary-heavy</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="106" t="inlineStr">
+      <c r="B13" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — NEW ($/yr)</t>
         </is>
@@ -3563,14 +5259,14 @@
       <c r="E13" s="47" t="n">
         <v>60000</v>
       </c>
-      <c r="G13" s="42" t="inlineStr">
+      <c r="G13" s="135" t="inlineStr">
         <is>
           <t>reduced base, upside from commission</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="106" t="inlineStr">
+      <c r="B14" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  James commission — NEW (% of signed value)</t>
         </is>
@@ -3578,14 +5274,14 @@
       <c r="E14" s="48" t="n">
         <v>0.01</v>
       </c>
-      <c r="G14" s="42" t="inlineStr">
+      <c r="G14" s="135" t="inlineStr">
         <is>
           <t>growth commission</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="106" t="inlineStr">
+      <c r="B15" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Number of sales reps</t>
         </is>
@@ -3593,10 +5289,10 @@
       <c r="E15" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="42" t="inlineStr"/>
+      <c r="G15" s="135" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="106" t="inlineStr">
+      <c r="B16" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rep base — OLD ($/yr each)</t>
         </is>
@@ -3604,10 +5300,10 @@
       <c r="E16" s="46" t="n">
         <v>60000</v>
       </c>
-      <c r="G16" s="42" t="inlineStr"/>
+      <c r="G16" s="135" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="106" t="inlineStr">
+      <c r="B17" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rep base — NEW ($/yr each)</t>
         </is>
@@ -3615,10 +5311,10 @@
       <c r="E17" s="47" t="n">
         <v>45000</v>
       </c>
-      <c r="G17" s="42" t="inlineStr"/>
+      <c r="G17" s="135" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="106" t="inlineStr">
+      <c r="B18" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Reps commission — NEW (% pooled)</t>
         </is>
@@ -3626,14 +5322,14 @@
       <c r="E18" s="48" t="n">
         <v>0.02</v>
       </c>
-      <c r="G18" s="42" t="inlineStr">
+      <c r="G18" s="135" t="inlineStr">
         <is>
           <t>across all reps, of signed value</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="106" t="inlineStr">
+      <c r="B19" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case manager loaded comp ($/yr)</t>
         </is>
@@ -3641,14 +5337,14 @@
       <c r="E19" s="84" t="n">
         <v>75000</v>
       </c>
-      <c r="G19" s="42" t="inlineStr">
+      <c r="G19" s="135" t="inlineStr">
         <is>
           <t>delivery cost per manager FTE</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="106" t="inlineStr">
+      <c r="B20" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead — fixed ($/yr)</t>
         </is>
@@ -3656,14 +5352,14 @@
       <c r="E20" s="84" t="n">
         <v>300000</v>
       </c>
-      <c r="G20" s="42" t="inlineStr">
+      <c r="G20" s="135" t="inlineStr">
         <is>
           <t>rent, software, admin</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="106" t="inlineStr">
+      <c r="B21" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead — variable (% of collected rev)</t>
         </is>
@@ -3671,14 +5367,14 @@
       <c r="E21" s="44" t="n">
         <v>0.3</v>
       </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="G21" s="135" t="inlineStr">
         <is>
           <t>marketing / lead-gen scales with revenue</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="91" t="inlineStr">
+      <c r="B23" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve">  ANNUAL RUN-RATE P&amp;L</t>
         </is>
@@ -3690,12 +5386,12 @@
           <t>Line</t>
         </is>
       </c>
-      <c r="E24" s="53" t="inlineStr">
+      <c r="E24" s="130" t="inlineStr">
         <is>
           <t>OLD comp</t>
         </is>
       </c>
-      <c r="G24" s="54" t="inlineStr">
+      <c r="G24" s="131" t="inlineStr">
         <is>
           <t>NEW comp</t>
         </is>
@@ -3707,187 +5403,187 @@
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="B25" s="106" t="inlineStr">
+      <c r="B25" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Intake (cases/week)</t>
         </is>
       </c>
-      <c r="E25" s="55">
+      <c r="E25" s="157">
         <f>E10</f>
         <v/>
       </c>
-      <c r="G25" s="55">
+      <c r="G25" s="157">
         <f>E11</f>
         <v/>
       </c>
-      <c r="H25" s="42" t="inlineStr">
+      <c r="H25" s="135" t="inlineStr">
         <is>
           <t>behavioral: new comp lifts volume</t>
         </is>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="B26" s="106" t="inlineStr">
+      <c r="B26" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Annual signed case value</t>
         </is>
       </c>
-      <c r="E26" s="94">
+      <c r="E26" s="153">
         <f>(E10*52*E6)</f>
         <v/>
       </c>
-      <c r="G26" s="94">
+      <c r="G26" s="153">
         <f>(E11*52*E6)</f>
         <v/>
       </c>
-      <c r="H26" s="42" t="inlineStr">
+      <c r="H26" s="135" t="inlineStr">
         <is>
           <t>cases/wk × 52 × case value</t>
         </is>
       </c>
     </row>
     <row r="27" ht="19" customHeight="1">
-      <c r="B27" s="106" t="inlineStr">
+      <c r="B27" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Collected revenue</t>
         </is>
       </c>
-      <c r="E27" s="94">
+      <c r="E27" s="153">
         <f>(E10*52*E6)*E9</f>
         <v/>
       </c>
-      <c r="G27" s="94">
+      <c r="G27" s="153">
         <f>(E11*52*E6)*E9</f>
         <v/>
       </c>
-      <c r="H27" s="42" t="inlineStr">
+      <c r="H27" s="135" t="inlineStr">
         <is>
           <t>signed × collection rate</t>
         </is>
       </c>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="B28" s="106" t="inlineStr">
+      <c r="B28" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case managers required (FTE)</t>
         </is>
       </c>
-      <c r="E28" s="55">
+      <c r="E28" s="157">
         <f>(E10*52*(E7/12))/E8</f>
         <v/>
       </c>
-      <c r="G28" s="55">
+      <c r="G28" s="157">
         <f>(E11*52*(E7/12))/E8</f>
         <v/>
       </c>
-      <c r="H28" s="42" t="inlineStr">
+      <c r="H28" s="135" t="inlineStr">
         <is>
           <t>active cases ÷ max per mgr</t>
         </is>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="B29" s="106" t="inlineStr">
+      <c r="B29" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case manager cost</t>
         </is>
       </c>
-      <c r="E29" s="94">
+      <c r="E29" s="153">
         <f>-((E10*52*(E7/12))/E8*E19)</f>
         <v/>
       </c>
-      <c r="G29" s="94">
+      <c r="G29" s="153">
         <f>-((E11*52*(E7/12))/E8*E19)</f>
         <v/>
       </c>
-      <c r="H29" s="42" t="inlineStr">
+      <c r="H29" s="135" t="inlineStr">
         <is>
           <t>required FTE × loaded comp</t>
         </is>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="B30" s="106" t="inlineStr">
+      <c r="B30" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  James pay</t>
         </is>
       </c>
-      <c r="E30" s="94">
+      <c r="E30" s="153">
         <f>-E12</f>
         <v/>
       </c>
-      <c r="G30" s="94">
+      <c r="G30" s="153">
         <f>-(E13+E14*(E11*52*E6))</f>
         <v/>
       </c>
-      <c r="H30" s="42" t="inlineStr">
+      <c r="H30" s="135" t="inlineStr">
         <is>
           <t>OLD base  |  NEW base + commission</t>
         </is>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="106" t="inlineStr">
+      <c r="B31" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sales reps pay</t>
         </is>
       </c>
-      <c r="E31" s="94">
+      <c r="E31" s="153">
         <f>-(E15*E16)</f>
         <v/>
       </c>
-      <c r="G31" s="94">
+      <c r="G31" s="153">
         <f>-(E15*E17+E18*(E11*52*E6))</f>
         <v/>
       </c>
-      <c r="H31" s="42" t="inlineStr">
+      <c r="H31" s="135" t="inlineStr">
         <is>
           <t>OLD base  |  NEW base + pooled commission</t>
         </is>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="B32" s="106" t="inlineStr">
+      <c r="B32" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  MG&amp;A overhead</t>
         </is>
       </c>
-      <c r="E32" s="94">
+      <c r="E32" s="153">
         <f>-(E20+E21*((E10*52*E6)*E9))</f>
         <v/>
       </c>
-      <c r="G32" s="94">
+      <c r="G32" s="153">
         <f>-(E20+E21*((E11*52*E6)*E9))</f>
         <v/>
       </c>
-      <c r="H32" s="42" t="inlineStr">
+      <c r="H32" s="135" t="inlineStr">
         <is>
           <t>fixed + variable % of collected rev</t>
         </is>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="101" t="inlineStr">
+      <c r="B33" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  NET PROFIT</t>
         </is>
       </c>
-      <c r="E33" s="99">
+      <c r="E33" s="143">
         <f>(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
         <v/>
       </c>
-      <c r="G33" s="99">
+      <c r="G33" s="143">
         <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))</f>
         <v/>
       </c>
-      <c r="H33" s="42" t="inlineStr">
+      <c r="H33" s="135" t="inlineStr">
         <is>
           <t>collected rev − all costs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="19" customHeight="1">
-      <c r="B34" s="101" t="inlineStr">
+      <c r="B34" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Net margin</t>
         </is>
@@ -3900,10 +5596,10 @@
         <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))/((E11*52*E6)*E9)</f>
         <v/>
       </c>
-      <c r="H34" s="42" t="inlineStr"/>
+      <c r="H34" s="135" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="112" t="inlineStr">
+      <c r="B36" s="144" t="inlineStr">
         <is>
           <t xml:space="preserve">  PROFITABILITY IMPACT OF THE NEW COMP MODEL</t>
         </is>
@@ -3915,11 +5611,11 @@
           <t xml:space="preserve">  Δ Collected revenue (new − old)</t>
         </is>
       </c>
-      <c r="E37" s="94">
+      <c r="E37" s="153">
         <f>((E11*52*E6)*E9)-((E10*52*E6)*E9)</f>
         <v/>
       </c>
-      <c r="G37" s="103" t="inlineStr">
+      <c r="G37" s="149" t="inlineStr">
         <is>
           <t>the growth the incentive unlocks</t>
         </is>
@@ -3931,11 +5627,11 @@
           <t xml:space="preserve">  Δ Selling comp cost (new − old)</t>
         </is>
       </c>
-      <c r="E38" s="94">
+      <c r="E38" s="153">
         <f>-(((E13+E14*(E11*52*E6))+(E15*E17+E18*(E11*52*E6)))-(E12+(E15*E16)))</f>
         <v/>
       </c>
-      <c r="G38" s="103" t="inlineStr">
+      <c r="G38" s="149" t="inlineStr">
         <is>
           <t>extra commission the firm pays out</t>
         </is>
@@ -3951,7 +5647,7 @@
         <f>(((E11*52*E6)*E9)-((E11*52*(E7/12))/E8*E19)-(E13+E14*(E11*52*E6))-(E15*E17+E18*(E11*52*E6))-(E20+E21*((E11*52*E6)*E9)))-(((E10*52*E6)*E9)-((E10*52*(E7/12))/E8*E19)-E12-(E15*E16)-(E20+E21*((E10*52*E6)*E9)))</f>
         <v/>
       </c>
-      <c r="G39" s="103" t="inlineStr">
+      <c r="G39" s="149" t="inlineStr">
         <is>
           <t>bottom-line effect of switching</t>
         </is>
@@ -3979,7 +5675,7 @@
       <c r="H42" s="36" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="B44" s="91" t="inlineStr">
+      <c r="B44" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
         </is>
@@ -4095,7 +5791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C8961E"/>
@@ -4129,7 +5825,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="101" t="inlineStr">
+      <c r="B5" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — OLD</t>
         </is>
@@ -4138,7 +5834,7 @@
         <f>'Profitability'!E12</f>
         <v/>
       </c>
-      <c r="E5" s="101" t="inlineStr">
+      <c r="E5" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Target intake (cases/wk)</t>
         </is>
@@ -4149,18 +5845,18 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="101" t="inlineStr">
+      <c r="B6" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  James base — NEW</t>
         </is>
       </c>
-      <c r="C6" s="69">
+      <c r="C6" s="137">
         <f>'Profitability'!E13</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="101" t="inlineStr">
+      <c r="B7" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Commission % (signed value)</t>
         </is>
@@ -4171,7 +5867,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="101" t="inlineStr">
+      <c r="B8" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Case value</t>
         </is>
@@ -4209,14 +5905,14 @@
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="55" t="n">
+      <c r="B12" s="157" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="94">
+      <c r="C12" s="153">
         <f>B12*52*$C$8</f>
         <v/>
       </c>
-      <c r="D12" s="94">
+      <c r="D12" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4224,20 +5920,20 @@
         <f>$C$6+$C$7*C12</f>
         <v/>
       </c>
-      <c r="F12" s="94">
+      <c r="F12" s="153">
         <f>E12-D12</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="55" t="n">
+      <c r="B13" s="157" t="n">
         <v>2.5</v>
       </c>
-      <c r="C13" s="94">
+      <c r="C13" s="153">
         <f>B13*52*$C$8</f>
         <v/>
       </c>
-      <c r="D13" s="94">
+      <c r="D13" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4245,20 +5941,20 @@
         <f>$C$6+$C$7*C13</f>
         <v/>
       </c>
-      <c r="F13" s="94">
+      <c r="F13" s="153">
         <f>E13-D13</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="55" t="n">
+      <c r="B14" s="157" t="n">
         <v>5</v>
       </c>
-      <c r="C14" s="94">
+      <c r="C14" s="153">
         <f>B14*52*$C$8</f>
         <v/>
       </c>
-      <c r="D14" s="94">
+      <c r="D14" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4266,20 +5962,20 @@
         <f>$C$6+$C$7*C14</f>
         <v/>
       </c>
-      <c r="F14" s="94">
+      <c r="F14" s="153">
         <f>E14-D14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="55" t="n">
+      <c r="B15" s="157" t="n">
         <v>7.5</v>
       </c>
-      <c r="C15" s="94">
+      <c r="C15" s="153">
         <f>B15*52*$C$8</f>
         <v/>
       </c>
-      <c r="D15" s="94">
+      <c r="D15" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4287,20 +5983,20 @@
         <f>$C$6+$C$7*C15</f>
         <v/>
       </c>
-      <c r="F15" s="94">
+      <c r="F15" s="153">
         <f>E15-D15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="55" t="n">
+      <c r="B16" s="157" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="94">
+      <c r="C16" s="153">
         <f>B16*52*$C$8</f>
         <v/>
       </c>
-      <c r="D16" s="94">
+      <c r="D16" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4308,20 +6004,20 @@
         <f>$C$6+$C$7*C16</f>
         <v/>
       </c>
-      <c r="F16" s="94">
+      <c r="F16" s="153">
         <f>E16-D16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="55" t="n">
+      <c r="B17" s="157" t="n">
         <v>12.5</v>
       </c>
-      <c r="C17" s="94">
+      <c r="C17" s="153">
         <f>B17*52*$C$8</f>
         <v/>
       </c>
-      <c r="D17" s="94">
+      <c r="D17" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4329,20 +6025,20 @@
         <f>$C$6+$C$7*C17</f>
         <v/>
       </c>
-      <c r="F17" s="94">
+      <c r="F17" s="153">
         <f>E17-D17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="55" t="n">
+      <c r="B18" s="157" t="n">
         <v>15</v>
       </c>
-      <c r="C18" s="94">
+      <c r="C18" s="153">
         <f>B18*52*$C$8</f>
         <v/>
       </c>
-      <c r="D18" s="94">
+      <c r="D18" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4350,20 +6046,20 @@
         <f>$C$6+$C$7*C18</f>
         <v/>
       </c>
-      <c r="F18" s="94">
+      <c r="F18" s="153">
         <f>E18-D18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="B19" s="55" t="n">
+      <c r="B19" s="157" t="n">
         <v>17.5</v>
       </c>
-      <c r="C19" s="94">
+      <c r="C19" s="153">
         <f>B19*52*$C$8</f>
         <v/>
       </c>
-      <c r="D19" s="94">
+      <c r="D19" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4371,20 +6067,20 @@
         <f>$C$6+$C$7*C19</f>
         <v/>
       </c>
-      <c r="F19" s="94">
+      <c r="F19" s="153">
         <f>E19-D19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="55" t="n">
+      <c r="B20" s="157" t="n">
         <v>20</v>
       </c>
-      <c r="C20" s="94">
+      <c r="C20" s="153">
         <f>B20*52*$C$8</f>
         <v/>
       </c>
-      <c r="D20" s="94">
+      <c r="D20" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4392,20 +6088,20 @@
         <f>$C$6+$C$7*C20</f>
         <v/>
       </c>
-      <c r="F20" s="94">
+      <c r="F20" s="153">
         <f>E20-D20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="55" t="n">
+      <c r="B21" s="157" t="n">
         <v>22.5</v>
       </c>
-      <c r="C21" s="94">
+      <c r="C21" s="153">
         <f>B21*52*$C$8</f>
         <v/>
       </c>
-      <c r="D21" s="94">
+      <c r="D21" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4413,7 +6109,7 @@
         <f>$C$6+$C$7*C21</f>
         <v/>
       </c>
-      <c r="F21" s="94">
+      <c r="F21" s="153">
         <f>E21-D21</f>
         <v/>
       </c>
@@ -4440,14 +6136,14 @@
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="55" t="n">
+      <c r="B23" s="157" t="n">
         <v>27.5</v>
       </c>
-      <c r="C23" s="94">
+      <c r="C23" s="153">
         <f>B23*52*$C$8</f>
         <v/>
       </c>
-      <c r="D23" s="94">
+      <c r="D23" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4455,20 +6151,20 @@
         <f>$C$6+$C$7*C23</f>
         <v/>
       </c>
-      <c r="F23" s="94">
+      <c r="F23" s="153">
         <f>E23-D23</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="55" t="n">
+      <c r="B24" s="157" t="n">
         <v>30</v>
       </c>
-      <c r="C24" s="94">
+      <c r="C24" s="153">
         <f>B24*52*$C$8</f>
         <v/>
       </c>
-      <c r="D24" s="94">
+      <c r="D24" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4476,20 +6172,20 @@
         <f>$C$6+$C$7*C24</f>
         <v/>
       </c>
-      <c r="F24" s="94">
+      <c r="F24" s="153">
         <f>E24-D24</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="55" t="n">
+      <c r="B25" s="157" t="n">
         <v>32.5</v>
       </c>
-      <c r="C25" s="94">
+      <c r="C25" s="153">
         <f>B25*52*$C$8</f>
         <v/>
       </c>
-      <c r="D25" s="94">
+      <c r="D25" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4497,20 +6193,20 @@
         <f>$C$6+$C$7*C25</f>
         <v/>
       </c>
-      <c r="F25" s="94">
+      <c r="F25" s="153">
         <f>E25-D25</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="55" t="n">
+      <c r="B26" s="157" t="n">
         <v>35</v>
       </c>
-      <c r="C26" s="94">
+      <c r="C26" s="153">
         <f>B26*52*$C$8</f>
         <v/>
       </c>
-      <c r="D26" s="94">
+      <c r="D26" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4518,20 +6214,20 @@
         <f>$C$6+$C$7*C26</f>
         <v/>
       </c>
-      <c r="F26" s="94">
+      <c r="F26" s="153">
         <f>E26-D26</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="55" t="n">
+      <c r="B27" s="157" t="n">
         <v>37.5</v>
       </c>
-      <c r="C27" s="94">
+      <c r="C27" s="153">
         <f>B27*52*$C$8</f>
         <v/>
       </c>
-      <c r="D27" s="94">
+      <c r="D27" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4539,20 +6235,20 @@
         <f>$C$6+$C$7*C27</f>
         <v/>
       </c>
-      <c r="F27" s="94">
+      <c r="F27" s="153">
         <f>E27-D27</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="55" t="n">
+      <c r="B28" s="157" t="n">
         <v>40</v>
       </c>
-      <c r="C28" s="94">
+      <c r="C28" s="153">
         <f>B28*52*$C$8</f>
         <v/>
       </c>
-      <c r="D28" s="94">
+      <c r="D28" s="153">
         <f>$C$5</f>
         <v/>
       </c>
@@ -4560,7 +6256,7 @@
         <f>$C$6+$C$7*C28</f>
         <v/>
       </c>
-      <c r="F28" s="94">
+      <c r="F28" s="153">
         <f>E28-D28</f>
         <v/>
       </c>
@@ -4602,7 +6298,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B3402E"/>
@@ -4641,7 +6337,7 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="82" t="inlineStr">
+      <c r="B5" s="119" t="inlineStr">
         <is>
           <t xml:space="preserve">  DRIVERS (linked from Profitability / Capacity Lite; yellow = editable)</t>
         </is>
@@ -4801,7 +6497,7 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="91" t="inlineStr">
+      <c r="B21" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve">  18-MONTH CASH PROJECTION</t>
         </is>
@@ -4860,10 +6556,10 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="93" t="n">
+      <c r="B23" s="155" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="94">
+      <c r="C23" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -4879,11 +6575,11 @@
         <f>E23*F18</f>
         <v/>
       </c>
-      <c r="G23" s="94">
+      <c r="G23" s="153">
         <f>E23/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H23" s="94">
+      <c r="H23" s="153">
         <f>F13+F16+F17*F23</f>
         <v/>
       </c>
@@ -4891,7 +6587,7 @@
         <f>F23-D23-G23-H23</f>
         <v/>
       </c>
-      <c r="J23" s="99">
+      <c r="J23" s="143">
         <f>F6+I23</f>
         <v/>
       </c>
@@ -4901,10 +6597,10 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="B24" s="93" t="n">
+      <c r="B24" s="155" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="94">
+      <c r="C24" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -4920,11 +6616,11 @@
         <f>E24*F18</f>
         <v/>
       </c>
-      <c r="G24" s="94">
+      <c r="G24" s="153">
         <f>E24/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H24" s="94">
+      <c r="H24" s="153">
         <f>F13+F16+F17*F24</f>
         <v/>
       </c>
@@ -4932,7 +6628,7 @@
         <f>F24-D24-G24-H24</f>
         <v/>
       </c>
-      <c r="J24" s="99">
+      <c r="J24" s="143">
         <f>J23+I24</f>
         <v/>
       </c>
@@ -4942,10 +6638,10 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="B25" s="93" t="n">
+      <c r="B25" s="155" t="n">
         <v>3</v>
       </c>
-      <c r="C25" s="94">
+      <c r="C25" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -4961,11 +6657,11 @@
         <f>E25*F18</f>
         <v/>
       </c>
-      <c r="G25" s="94">
+      <c r="G25" s="153">
         <f>E25/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H25" s="94">
+      <c r="H25" s="153">
         <f>F13+F16+F17*F25</f>
         <v/>
       </c>
@@ -4973,7 +6669,7 @@
         <f>F25-D25-G25-H25</f>
         <v/>
       </c>
-      <c r="J25" s="99">
+      <c r="J25" s="143">
         <f>J24+I25</f>
         <v/>
       </c>
@@ -4983,10 +6679,10 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="B26" s="93" t="n">
+      <c r="B26" s="155" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="94">
+      <c r="C26" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5002,11 +6698,11 @@
         <f>E26*F18</f>
         <v/>
       </c>
-      <c r="G26" s="94">
+      <c r="G26" s="153">
         <f>E26/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H26" s="94">
+      <c r="H26" s="153">
         <f>F13+F16+F17*F26</f>
         <v/>
       </c>
@@ -5014,7 +6710,7 @@
         <f>F26-D26-G26-H26</f>
         <v/>
       </c>
-      <c r="J26" s="99">
+      <c r="J26" s="143">
         <f>J25+I26</f>
         <v/>
       </c>
@@ -5024,10 +6720,10 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="B27" s="93" t="n">
+      <c r="B27" s="155" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="94">
+      <c r="C27" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5043,11 +6739,11 @@
         <f>E27*F18</f>
         <v/>
       </c>
-      <c r="G27" s="94">
+      <c r="G27" s="153">
         <f>E27/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H27" s="94">
+      <c r="H27" s="153">
         <f>F13+F16+F17*F27</f>
         <v/>
       </c>
@@ -5055,7 +6751,7 @@
         <f>F27-D27-G27-H27</f>
         <v/>
       </c>
-      <c r="J27" s="99">
+      <c r="J27" s="143">
         <f>J26+I27</f>
         <v/>
       </c>
@@ -5065,10 +6761,10 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="B28" s="93" t="n">
+      <c r="B28" s="155" t="n">
         <v>6</v>
       </c>
-      <c r="C28" s="94">
+      <c r="C28" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5084,11 +6780,11 @@
         <f>E28*F18</f>
         <v/>
       </c>
-      <c r="G28" s="94">
+      <c r="G28" s="153">
         <f>E28/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H28" s="94">
+      <c r="H28" s="153">
         <f>F13+F16+F17*F28</f>
         <v/>
       </c>
@@ -5096,7 +6792,7 @@
         <f>F28-D28-G28-H28</f>
         <v/>
       </c>
-      <c r="J28" s="99">
+      <c r="J28" s="143">
         <f>J27+I28</f>
         <v/>
       </c>
@@ -5106,10 +6802,10 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="B29" s="93" t="n">
+      <c r="B29" s="155" t="n">
         <v>7</v>
       </c>
-      <c r="C29" s="94">
+      <c r="C29" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5125,11 +6821,11 @@
         <f>E29*F18</f>
         <v/>
       </c>
-      <c r="G29" s="94">
+      <c r="G29" s="153">
         <f>E29/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H29" s="94">
+      <c r="H29" s="153">
         <f>F13+F16+F17*F29</f>
         <v/>
       </c>
@@ -5137,7 +6833,7 @@
         <f>F29-D29-G29-H29</f>
         <v/>
       </c>
-      <c r="J29" s="99">
+      <c r="J29" s="143">
         <f>J28+I29</f>
         <v/>
       </c>
@@ -5147,10 +6843,10 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="93" t="n">
+      <c r="B30" s="155" t="n">
         <v>8</v>
       </c>
-      <c r="C30" s="94">
+      <c r="C30" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5166,11 +6862,11 @@
         <f>E30*F18</f>
         <v/>
       </c>
-      <c r="G30" s="94">
+      <c r="G30" s="153">
         <f>E30/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H30" s="94">
+      <c r="H30" s="153">
         <f>F13+F16+F17*F30</f>
         <v/>
       </c>
@@ -5178,7 +6874,7 @@
         <f>F30-D30-G30-H30</f>
         <v/>
       </c>
-      <c r="J30" s="99">
+      <c r="J30" s="143">
         <f>J29+I30</f>
         <v/>
       </c>
@@ -5188,10 +6884,10 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="93" t="n">
+      <c r="B31" s="155" t="n">
         <v>9</v>
       </c>
-      <c r="C31" s="94">
+      <c r="C31" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5207,11 +6903,11 @@
         <f>E31*F18</f>
         <v/>
       </c>
-      <c r="G31" s="94">
+      <c r="G31" s="153">
         <f>E31/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H31" s="94">
+      <c r="H31" s="153">
         <f>F13+F16+F17*F31</f>
         <v/>
       </c>
@@ -5219,7 +6915,7 @@
         <f>F31-D31-G31-H31</f>
         <v/>
       </c>
-      <c r="J31" s="99">
+      <c r="J31" s="143">
         <f>J30+I31</f>
         <v/>
       </c>
@@ -5229,10 +6925,10 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="B32" s="93" t="n">
+      <c r="B32" s="155" t="n">
         <v>10</v>
       </c>
-      <c r="C32" s="94">
+      <c r="C32" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5248,11 +6944,11 @@
         <f>E32*F18</f>
         <v/>
       </c>
-      <c r="G32" s="94">
+      <c r="G32" s="153">
         <f>E32/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H32" s="94">
+      <c r="H32" s="153">
         <f>F13+F16+F17*F32</f>
         <v/>
       </c>
@@ -5260,7 +6956,7 @@
         <f>F32-D32-G32-H32</f>
         <v/>
       </c>
-      <c r="J32" s="99">
+      <c r="J32" s="143">
         <f>J31+I32</f>
         <v/>
       </c>
@@ -5270,10 +6966,10 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="B33" s="93" t="n">
+      <c r="B33" s="155" t="n">
         <v>11</v>
       </c>
-      <c r="C33" s="94">
+      <c r="C33" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5289,11 +6985,11 @@
         <f>E33*F18</f>
         <v/>
       </c>
-      <c r="G33" s="94">
+      <c r="G33" s="153">
         <f>E33/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H33" s="94">
+      <c r="H33" s="153">
         <f>F13+F16+F17*F33</f>
         <v/>
       </c>
@@ -5301,7 +6997,7 @@
         <f>F33-D33-G33-H33</f>
         <v/>
       </c>
-      <c r="J33" s="99">
+      <c r="J33" s="143">
         <f>J32+I33</f>
         <v/>
       </c>
@@ -5311,10 +7007,10 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="B34" s="93" t="n">
+      <c r="B34" s="155" t="n">
         <v>12</v>
       </c>
-      <c r="C34" s="94">
+      <c r="C34" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5330,11 +7026,11 @@
         <f>E34*F18</f>
         <v/>
       </c>
-      <c r="G34" s="94">
+      <c r="G34" s="153">
         <f>E34/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H34" s="94">
+      <c r="H34" s="153">
         <f>F13+F16+F17*F34</f>
         <v/>
       </c>
@@ -5342,7 +7038,7 @@
         <f>F34-D34-G34-H34</f>
         <v/>
       </c>
-      <c r="J34" s="99">
+      <c r="J34" s="143">
         <f>J33+I34</f>
         <v/>
       </c>
@@ -5352,10 +7048,10 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="B35" s="93" t="n">
+      <c r="B35" s="155" t="n">
         <v>13</v>
       </c>
-      <c r="C35" s="94">
+      <c r="C35" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5371,11 +7067,11 @@
         <f>E35*F18</f>
         <v/>
       </c>
-      <c r="G35" s="94">
+      <c r="G35" s="153">
         <f>E35/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H35" s="94">
+      <c r="H35" s="153">
         <f>F13+F16+F17*F35</f>
         <v/>
       </c>
@@ -5383,7 +7079,7 @@
         <f>F35-D35-G35-H35</f>
         <v/>
       </c>
-      <c r="J35" s="99">
+      <c r="J35" s="143">
         <f>J34+I35</f>
         <v/>
       </c>
@@ -5393,10 +7089,10 @@
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
-      <c r="B36" s="93" t="n">
+      <c r="B36" s="155" t="n">
         <v>14</v>
       </c>
-      <c r="C36" s="94">
+      <c r="C36" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5412,11 +7108,11 @@
         <f>E36*F18</f>
         <v/>
       </c>
-      <c r="G36" s="94">
+      <c r="G36" s="153">
         <f>E36/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H36" s="94">
+      <c r="H36" s="153">
         <f>F13+F16+F17*F36</f>
         <v/>
       </c>
@@ -5424,7 +7120,7 @@
         <f>F36-D36-G36-H36</f>
         <v/>
       </c>
-      <c r="J36" s="99">
+      <c r="J36" s="143">
         <f>J35+I36</f>
         <v/>
       </c>
@@ -5434,10 +7130,10 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="B37" s="93" t="n">
+      <c r="B37" s="155" t="n">
         <v>15</v>
       </c>
-      <c r="C37" s="94">
+      <c r="C37" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5453,11 +7149,11 @@
         <f>E37*F18</f>
         <v/>
       </c>
-      <c r="G37" s="94">
+      <c r="G37" s="153">
         <f>E37/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H37" s="94">
+      <c r="H37" s="153">
         <f>F13+F16+F17*F37</f>
         <v/>
       </c>
@@ -5465,7 +7161,7 @@
         <f>F37-D37-G37-H37</f>
         <v/>
       </c>
-      <c r="J37" s="99">
+      <c r="J37" s="143">
         <f>J36+I37</f>
         <v/>
       </c>
@@ -5475,10 +7171,10 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="93" t="n">
+      <c r="B38" s="155" t="n">
         <v>16</v>
       </c>
-      <c r="C38" s="94">
+      <c r="C38" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5494,11 +7190,11 @@
         <f>E38*F18</f>
         <v/>
       </c>
-      <c r="G38" s="94">
+      <c r="G38" s="153">
         <f>E38/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H38" s="94">
+      <c r="H38" s="153">
         <f>F13+F16+F17*F38</f>
         <v/>
       </c>
@@ -5506,7 +7202,7 @@
         <f>F38-D38-G38-H38</f>
         <v/>
       </c>
-      <c r="J38" s="99">
+      <c r="J38" s="143">
         <f>J37+I38</f>
         <v/>
       </c>
@@ -5516,10 +7212,10 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="B39" s="93" t="n">
+      <c r="B39" s="155" t="n">
         <v>17</v>
       </c>
-      <c r="C39" s="94">
+      <c r="C39" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5535,11 +7231,11 @@
         <f>E39*F18</f>
         <v/>
       </c>
-      <c r="G39" s="94">
+      <c r="G39" s="153">
         <f>E39/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H39" s="94">
+      <c r="H39" s="153">
         <f>F13+F16+F17*F39</f>
         <v/>
       </c>
@@ -5547,7 +7243,7 @@
         <f>F39-D39-G39-H39</f>
         <v/>
       </c>
-      <c r="J39" s="99">
+      <c r="J39" s="143">
         <f>J38+I39</f>
         <v/>
       </c>
@@ -5557,10 +7253,10 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="B40" s="93" t="n">
+      <c r="B40" s="155" t="n">
         <v>18</v>
       </c>
-      <c r="C40" s="94">
+      <c r="C40" s="153">
         <f>F8*F9</f>
         <v/>
       </c>
@@ -5576,11 +7272,11 @@
         <f>E40*F18</f>
         <v/>
       </c>
-      <c r="G40" s="94">
+      <c r="G40" s="153">
         <f>E40/F14*F15/12</f>
         <v/>
       </c>
-      <c r="H40" s="94">
+      <c r="H40" s="153">
         <f>F13+F16+F17*F40</f>
         <v/>
       </c>
@@ -5588,7 +7284,7 @@
         <f>F40-D40-G40-H40</f>
         <v/>
       </c>
-      <c r="J40" s="99">
+      <c r="J40" s="143">
         <f>J39+I40</f>
         <v/>
       </c>
@@ -5598,7 +7294,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="101" t="inlineStr">
+      <c r="B42" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cash-flow trough (min cumulative)</t>
         </is>
@@ -5607,14 +7303,14 @@
         <f>MIN(J23:J40)</f>
         <v/>
       </c>
-      <c r="G42" s="103" t="inlineStr">
+      <c r="G42" s="149" t="inlineStr">
         <is>
           <t>lowest your cash gets during the ramp</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="101" t="inlineStr">
+      <c r="B43" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Month-1 cash vs run-rate profit gap</t>
         </is>
@@ -5623,7 +7319,7 @@
         <f>K23-F23</f>
         <v/>
       </c>
-      <c r="G43" s="103" t="inlineStr">
+      <c r="G43" s="149" t="inlineStr">
         <is>
           <t>collections shortfall vs steady-state in month 1</t>
         </is>
@@ -5705,7 +7401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001B2A4A"/>
@@ -5725,7 +7421,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="105" t="inlineStr">
+      <c r="B2" s="118" t="inlineStr">
         <is>
           <t>COMP OPTIMIZER  ·  Highest James Rate the Firm Can Afford</t>
         </is>
@@ -5739,14 +7435,14 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="82" t="inlineStr">
+      <c r="B5" s="119" t="inlineStr">
         <is>
           <t xml:space="preserve">  INPUT</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="106" t="inlineStr">
+      <c r="B6" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Target net margin (floor)</t>
         </is>
@@ -5765,46 +7461,46 @@
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="B8" s="91" t="inlineStr">
+      <c r="B8" s="128" t="inlineStr">
         <is>
           <t xml:space="preserve">  RESULTS</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="106" t="inlineStr">
+      <c r="B9" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Firm net profit — OLD model</t>
         </is>
       </c>
-      <c r="C9" s="94">
+      <c r="C9" s="153">
         <f>((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)))</f>
         <v/>
       </c>
-      <c r="D9" s="103" t="inlineStr">
+      <c r="D9" s="149" t="inlineStr">
         <is>
           <t>the floor to beat</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="106" t="inlineStr">
+      <c r="B10" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Firm net profit — NEW (at current James %)</t>
         </is>
       </c>
-      <c r="C10" s="94">
+      <c r="C10" s="153">
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-'Profitability'!E14*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="D10" s="103" t="inlineStr">
+      <c r="D10" s="149" t="inlineStr">
         <is>
           <t>with James commission applied</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="101" t="inlineStr">
+      <c r="B11" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Max James % — stay ACCRETIVE vs old</t>
         </is>
@@ -5813,14 +7509,14 @@
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))))/('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="D11" s="103" t="inlineStr">
+      <c r="D11" s="149" t="inlineStr">
         <is>
           <t>above this, firm earns less than old model</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="101" t="inlineStr">
+      <c r="B12" s="120" t="inlineStr">
         <is>
           <t xml:space="preserve">  Max James % — hold target margin</t>
         </is>
@@ -5829,14 +7525,14 @@
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-C6*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9))/('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="D12" s="103" t="inlineStr">
+      <c r="D12" s="149" t="inlineStr">
         <is>
           <t>above this, margin falls below the floor</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="106" t="inlineStr">
+      <c r="B13" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">  Headroom on James % (accretive − current)</t>
         </is>
@@ -5845,14 +7541,14 @@
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))))/('Profitability'!E11*52*'Profitability'!E6)-'Profitability'!E14</f>
         <v/>
       </c>
-      <c r="D13" s="103" t="inlineStr">
+      <c r="D13" s="149" t="inlineStr">
         <is>
           <t>how much room to raise his rate</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="112" t="inlineStr">
+      <c r="B15" s="144" t="inlineStr">
         <is>
           <t xml:space="preserve">  SENSITIVITY — James commission % vs firm profit &amp; his pay</t>
         </is>
@@ -5894,7 +7590,7 @@
       <c r="B17" s="115" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="116">
+      <c r="C17" s="156">
         <f>'Profitability'!E13+B17*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -5902,11 +7598,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E17" s="117">
+      <c r="E17" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F17" s="93">
+      <c r="F17" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B17*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -5919,7 +7615,7 @@
       <c r="B18" s="115" t="n">
         <v>0.005</v>
       </c>
-      <c r="C18" s="116">
+      <c r="C18" s="156">
         <f>'Profitability'!E13+B18*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -5927,11 +7623,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E18" s="117">
+      <c r="E18" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F18" s="93">
+      <c r="F18" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B18*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -5944,7 +7640,7 @@
       <c r="B19" s="115" t="n">
         <v>0.01</v>
       </c>
-      <c r="C19" s="116">
+      <c r="C19" s="156">
         <f>'Profitability'!E13+B19*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -5952,11 +7648,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E19" s="117">
+      <c r="E19" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F19" s="93">
+      <c r="F19" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B19*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -5969,7 +7665,7 @@
       <c r="B20" s="115" t="n">
         <v>0.015</v>
       </c>
-      <c r="C20" s="116">
+      <c r="C20" s="156">
         <f>'Profitability'!E13+B20*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -5977,11 +7673,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E20" s="117">
+      <c r="E20" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F20" s="93">
+      <c r="F20" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B20*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -5994,7 +7690,7 @@
       <c r="B21" s="115" t="n">
         <v>0.02</v>
       </c>
-      <c r="C21" s="116">
+      <c r="C21" s="156">
         <f>'Profitability'!E13+B21*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6002,11 +7698,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E21" s="117">
+      <c r="E21" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F21" s="93">
+      <c r="F21" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B21*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6019,7 +7715,7 @@
       <c r="B22" s="115" t="n">
         <v>0.025</v>
       </c>
-      <c r="C22" s="116">
+      <c r="C22" s="156">
         <f>'Profitability'!E13+B22*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6027,11 +7723,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E22" s="117">
+      <c r="E22" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F22" s="93">
+      <c r="F22" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B22*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6044,7 +7740,7 @@
       <c r="B23" s="115" t="n">
         <v>0.03</v>
       </c>
-      <c r="C23" s="116">
+      <c r="C23" s="156">
         <f>'Profitability'!E13+B23*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6052,11 +7748,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E23" s="117">
+      <c r="E23" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F23" s="93">
+      <c r="F23" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B23*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6069,7 +7765,7 @@
       <c r="B24" s="115" t="n">
         <v>0.035</v>
       </c>
-      <c r="C24" s="116">
+      <c r="C24" s="156">
         <f>'Profitability'!E13+B24*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6077,11 +7773,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E24" s="117">
+      <c r="E24" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F24" s="93">
+      <c r="F24" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B24*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6094,7 +7790,7 @@
       <c r="B25" s="115" t="n">
         <v>0.04</v>
       </c>
-      <c r="C25" s="116">
+      <c r="C25" s="156">
         <f>'Profitability'!E13+B25*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6102,11 +7798,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E25" s="117">
+      <c r="E25" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F25" s="93">
+      <c r="F25" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B25*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6119,7 +7815,7 @@
       <c r="B26" s="115" t="n">
         <v>0.045</v>
       </c>
-      <c r="C26" s="116">
+      <c r="C26" s="156">
         <f>'Profitability'!E13+B26*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6127,11 +7823,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E26" s="117">
+      <c r="E26" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F26" s="93">
+      <c r="F26" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B26*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6144,7 +7840,7 @@
       <c r="B27" s="115" t="n">
         <v>0.05</v>
       </c>
-      <c r="C27" s="116">
+      <c r="C27" s="156">
         <f>'Profitability'!E13+B27*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6152,11 +7848,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E27" s="117">
+      <c r="E27" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F27" s="93">
+      <c r="F27" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B27*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6169,7 +7865,7 @@
       <c r="B28" s="115" t="n">
         <v>0.055</v>
       </c>
-      <c r="C28" s="116">
+      <c r="C28" s="156">
         <f>'Profitability'!E13+B28*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6177,11 +7873,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E28" s="117">
+      <c r="E28" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F28" s="93">
+      <c r="F28" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B28*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>
@@ -6194,7 +7890,7 @@
       <c r="B29" s="115" t="n">
         <v>0.06</v>
       </c>
-      <c r="C29" s="116">
+      <c r="C29" s="156">
         <f>'Profitability'!E13+B29*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
@@ -6202,11 +7898,11 @@
         <f>((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6)</f>
         <v/>
       </c>
-      <c r="E29" s="117">
+      <c r="E29" s="154">
         <f>(((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6))/(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)</f>
         <v/>
       </c>
-      <c r="F29" s="93">
+      <c r="F29" s="155">
         <f>IF((((('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E11*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E13-('Profitability'!E15*'Profitability'!E17+'Profitability'!E18*('Profitability'!E11*52*'Profitability'!E6))-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E11*52*'Profitability'!E6)*'Profitability'!E9)))-B29*('Profitability'!E11*52*'Profitability'!E6))&gt;=((('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9)-(('Profitability'!E10*52*('Profitability'!E7/12))/'Profitability'!E8*'Profitability'!E19)-'Profitability'!E12-('Profitability'!E15*'Profitability'!E16)-('Profitability'!E20+'Profitability'!E21*(('Profitability'!E10*52*'Profitability'!E6)*'Profitability'!E9))),"yes","no")</f>
         <v/>
       </c>

</xml_diff>